<commit_message>
Nuevos campos en implementación y verificación
</commit_message>
<xml_diff>
--- a/GestionAmbiental/wwwroot/ExcelTemplates/Inspecciones/JU-MAP-PRO-004.F01_Inspección_V01.xlsx
+++ b/GestionAmbiental/wwwroot/ExcelTemplates/Inspecciones/JU-MAP-PRO-004.F01_Inspección_V01.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Electrodata\Marcobre\Gestiona Marcobre\Marcobre-GestionAmbiental\GestionAmbiental\wwwroot\ExcelTemplates\Inspecciones\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5ED5E7A9-ADAA-4809-A8AC-73430D35C002}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C36B8806-8767-4E17-A45A-0A6D6753CADE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="813" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -45,284 +45,6 @@
 </workbook>
 </file>
 
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
-  <authors>
-    <author>Doris Janeth Sanchez Aiquipa</author>
-    <author>Olivia Valencia</author>
-    <author>Carlos Gabriel Mego Armas</author>
-  </authors>
-  <commentList>
-    <comment ref="H14" authorId="0" shapeId="0" xr:uid="{DB5F720A-040D-4386-9A42-C4230CB033DA}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Doris Janeth Sanchez Aiquipa:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Incluir la opción:
-Comité de SSO</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="P14" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0100-000002000000}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>SGA:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Ingresar la hora en formato de 24 horas.
-Ejem:
-18:39</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="S14" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0100-000003000000}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>SGA:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Ingresar la fecha en el siguiente formato:
-dd/mm/aaaa
-Ejm: 19/12/2019</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="V14" authorId="0" shapeId="0" xr:uid="{F827DDA6-5313-4978-9927-E5B8F5E7E1FF}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Doris Janeth Sanchez Aiquipa:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Que haya opción de colocar el nombre completo uno por uno, para que se puedan contabilizar para cumplimiento de los KPI</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="A25" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0100-000004000000}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>SGA:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Para el desarrollo de la inspección de MA, puede agenciarse del check list que en encuentra en la hoja "Check list Insp.Amb."</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C27" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0100-000005000000}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>SGA:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Seleccionar.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="L27" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0100-000006000000}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">SGA:
-</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Seleccionar.
-Puede visualizar todos los tipos de condición/acto subestándar para SSO y MA en la hoja Tablas.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="R27" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0100-000007000000}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">SGA:
-</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Seleccionar.</t>
-        </r>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Puede visualizar los niveles de riesgo de MA en la hoja "Nivel Riesgo MA", y los niveles de riesgo de Sso en la hoja " Nivel Riesgo SSO".</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="X27" authorId="2" shapeId="0" xr:uid="{00000000-0006-0000-0100-000008000000}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>SGA:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Durante la inspección, el responsable del área indica la fecha de cumplimiento, la cual debe estar validada por el Ing. Ambiental o el Ing. De SSO (según corresponda). Ésta debe ser lógica de acuerdo con el nivel de riesgo.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="Y27" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0100-000009000000}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>SGA:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Colocar  la evidencia del levantamiento de la observación (Fotografías). En caso de ser documentos, vídeos u otros deberá indicarse ver "nombre del archivo", estos archivos deberán colocarse dentro de la misma carpeta donde se encuentre el archivo de la inspección.</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="293">
   <si>
@@ -1234,7 +956,7 @@
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy;@"/>
     <numFmt numFmtId="165" formatCode="dd/mmm/yyyy;@"/>
   </numFmts>
-  <fonts count="23" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1257,19 +979,6 @@
       <b/>
       <sz val="10"/>
       <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
       <family val="2"/>
     </font>
     <font>
@@ -1621,7 +1330,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="0"/>
   </cellStyleXfs>
-  <cellXfs count="222">
+  <cellXfs count="224">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1630,19 +1339,19 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0" hidden="1"/>
     </xf>
@@ -1666,15 +1375,15 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0" hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0" hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0" hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
       <protection locked="0" hidden="1"/>
     </xf>
@@ -1682,7 +1391,7 @@
       <alignment vertical="center"/>
       <protection locked="0" hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
       <protection locked="0" hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
@@ -1694,10 +1403,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1718,15 +1427,15 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1783,15 +1492,15 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="1" applyBorder="1" applyAlignment="1">
@@ -1811,7 +1520,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1821,7 +1530,7 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1831,10 +1540,10 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1866,7 +1575,7 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1888,11 +1597,11 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1905,43 +1614,43 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0" hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0" hidden="1"/>
     </xf>
-    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0" hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
       <protection locked="0" hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
@@ -1976,8 +1685,140 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2012,29 +1853,32 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2054,12 +1898,6 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2087,122 +1925,11 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
@@ -2210,43 +1937,31 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="13" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="13" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="13" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="13" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -4040,7 +3755,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -4082,125 +3797,125 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:31" ht="20.65" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="131"/>
-      <c r="B1" s="132"/>
-      <c r="C1" s="132"/>
-      <c r="D1" s="132"/>
-      <c r="E1" s="132"/>
-      <c r="F1" s="132"/>
-      <c r="G1" s="133"/>
-      <c r="H1" s="165" t="s">
+      <c r="A1" s="175"/>
+      <c r="B1" s="176"/>
+      <c r="C1" s="176"/>
+      <c r="D1" s="176"/>
+      <c r="E1" s="176"/>
+      <c r="F1" s="176"/>
+      <c r="G1" s="177"/>
+      <c r="H1" s="129" t="s">
         <v>0</v>
       </c>
-      <c r="I1" s="166"/>
-      <c r="J1" s="166"/>
-      <c r="K1" s="166"/>
-      <c r="L1" s="166"/>
-      <c r="M1" s="166"/>
-      <c r="N1" s="166"/>
-      <c r="O1" s="166"/>
-      <c r="P1" s="166"/>
-      <c r="Q1" s="166"/>
-      <c r="R1" s="166"/>
-      <c r="S1" s="166"/>
-      <c r="T1" s="166"/>
-      <c r="U1" s="166"/>
-      <c r="V1" s="166"/>
-      <c r="W1" s="166"/>
-      <c r="X1" s="166"/>
-      <c r="Y1" s="166"/>
-      <c r="Z1" s="166"/>
-      <c r="AA1" s="167"/>
-      <c r="AB1" s="156"/>
-      <c r="AC1" s="157"/>
-      <c r="AD1" s="157"/>
-      <c r="AE1" s="158"/>
+      <c r="I1" s="130"/>
+      <c r="J1" s="130"/>
+      <c r="K1" s="130"/>
+      <c r="L1" s="130"/>
+      <c r="M1" s="130"/>
+      <c r="N1" s="130"/>
+      <c r="O1" s="130"/>
+      <c r="P1" s="130"/>
+      <c r="Q1" s="130"/>
+      <c r="R1" s="130"/>
+      <c r="S1" s="130"/>
+      <c r="T1" s="130"/>
+      <c r="U1" s="130"/>
+      <c r="V1" s="130"/>
+      <c r="W1" s="130"/>
+      <c r="X1" s="130"/>
+      <c r="Y1" s="130"/>
+      <c r="Z1" s="130"/>
+      <c r="AA1" s="131"/>
+      <c r="AB1" s="199"/>
+      <c r="AC1" s="200"/>
+      <c r="AD1" s="200"/>
+      <c r="AE1" s="201"/>
     </row>
     <row r="2" spans="1:31" ht="29.65" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="134"/>
-      <c r="B2" s="135"/>
-      <c r="C2" s="135"/>
-      <c r="D2" s="135"/>
-      <c r="E2" s="135"/>
-      <c r="F2" s="135"/>
-      <c r="G2" s="136"/>
+      <c r="A2" s="178"/>
+      <c r="B2" s="179"/>
+      <c r="C2" s="179"/>
+      <c r="D2" s="179"/>
+      <c r="E2" s="179"/>
+      <c r="F2" s="179"/>
+      <c r="G2" s="180"/>
       <c r="H2" s="68" t="s">
         <v>32</v>
       </c>
-      <c r="I2" s="168"/>
-      <c r="J2" s="168"/>
-      <c r="K2" s="168"/>
-      <c r="L2" s="168"/>
-      <c r="M2" s="168"/>
-      <c r="N2" s="168"/>
-      <c r="O2" s="169"/>
-      <c r="P2" s="191" t="s">
+      <c r="I2" s="132"/>
+      <c r="J2" s="132"/>
+      <c r="K2" s="132"/>
+      <c r="L2" s="132"/>
+      <c r="M2" s="132"/>
+      <c r="N2" s="132"/>
+      <c r="O2" s="133"/>
+      <c r="P2" s="187" t="s">
         <v>4</v>
       </c>
-      <c r="Q2" s="192"/>
-      <c r="R2" s="189">
+      <c r="Q2" s="188"/>
+      <c r="R2" s="185">
         <v>43831</v>
       </c>
-      <c r="S2" s="189"/>
-      <c r="T2" s="189"/>
-      <c r="U2" s="189"/>
-      <c r="V2" s="190"/>
+      <c r="S2" s="185"/>
+      <c r="T2" s="185"/>
+      <c r="U2" s="185"/>
+      <c r="V2" s="186"/>
       <c r="W2" s="123" t="s">
         <v>5</v>
       </c>
-      <c r="X2" s="148" t="s">
+      <c r="X2" s="193" t="s">
         <v>209</v>
       </c>
-      <c r="Y2" s="148"/>
-      <c r="Z2" s="148"/>
-      <c r="AA2" s="149"/>
-      <c r="AB2" s="159"/>
-      <c r="AC2" s="160"/>
-      <c r="AD2" s="160"/>
-      <c r="AE2" s="161"/>
+      <c r="Y2" s="193"/>
+      <c r="Z2" s="193"/>
+      <c r="AA2" s="194"/>
+      <c r="AB2" s="202"/>
+      <c r="AC2" s="203"/>
+      <c r="AD2" s="203"/>
+      <c r="AE2" s="204"/>
     </row>
     <row r="3" spans="1:31" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="137"/>
-      <c r="B3" s="138"/>
-      <c r="C3" s="138"/>
-      <c r="D3" s="138"/>
-      <c r="E3" s="138"/>
-      <c r="F3" s="138"/>
-      <c r="G3" s="139"/>
+      <c r="A3" s="181"/>
+      <c r="B3" s="182"/>
+      <c r="C3" s="182"/>
+      <c r="D3" s="182"/>
+      <c r="E3" s="182"/>
+      <c r="F3" s="182"/>
+      <c r="G3" s="183"/>
       <c r="H3" s="68" t="s">
         <v>7</v>
       </c>
-      <c r="I3" s="168"/>
-      <c r="J3" s="168"/>
-      <c r="K3" s="168"/>
-      <c r="L3" s="168"/>
-      <c r="M3" s="168"/>
-      <c r="N3" s="168"/>
-      <c r="O3" s="169"/>
-      <c r="P3" s="170" t="s">
+      <c r="I3" s="132"/>
+      <c r="J3" s="132"/>
+      <c r="K3" s="132"/>
+      <c r="L3" s="132"/>
+      <c r="M3" s="132"/>
+      <c r="N3" s="132"/>
+      <c r="O3" s="133"/>
+      <c r="P3" s="134" t="s">
         <v>26</v>
       </c>
-      <c r="Q3" s="171"/>
-      <c r="R3" s="129">
+      <c r="Q3" s="135"/>
+      <c r="R3" s="173">
         <v>1</v>
       </c>
-      <c r="S3" s="129"/>
-      <c r="T3" s="129"/>
-      <c r="U3" s="129"/>
-      <c r="V3" s="130"/>
-      <c r="W3" s="198" t="s">
+      <c r="S3" s="173"/>
+      <c r="T3" s="173"/>
+      <c r="U3" s="173"/>
+      <c r="V3" s="174"/>
+      <c r="W3" s="157" t="s">
         <v>6</v>
       </c>
-      <c r="X3" s="199"/>
-      <c r="Y3" s="196">
+      <c r="X3" s="158"/>
+      <c r="Y3" s="155">
         <v>43800</v>
       </c>
-      <c r="Z3" s="196"/>
-      <c r="AA3" s="197"/>
-      <c r="AB3" s="162"/>
-      <c r="AC3" s="163"/>
-      <c r="AD3" s="163"/>
-      <c r="AE3" s="164"/>
+      <c r="Z3" s="155"/>
+      <c r="AA3" s="156"/>
+      <c r="AB3" s="205"/>
+      <c r="AC3" s="206"/>
+      <c r="AD3" s="206"/>
+      <c r="AE3" s="207"/>
     </row>
     <row r="4" spans="1:31" ht="13.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="69"/>
@@ -4235,39 +3950,39 @@
       <c r="AE4" s="124"/>
     </row>
     <row r="5" spans="1:31" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="140" t="s">
+      <c r="A5" s="149" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="141"/>
-      <c r="C5" s="141"/>
-      <c r="D5" s="141"/>
-      <c r="E5" s="141"/>
-      <c r="F5" s="141"/>
-      <c r="G5" s="141"/>
-      <c r="H5" s="141"/>
-      <c r="I5" s="141"/>
-      <c r="J5" s="141"/>
-      <c r="K5" s="141"/>
-      <c r="L5" s="141"/>
-      <c r="M5" s="141"/>
-      <c r="N5" s="141"/>
-      <c r="O5" s="141"/>
-      <c r="P5" s="141"/>
-      <c r="Q5" s="141"/>
-      <c r="R5" s="141"/>
-      <c r="S5" s="141"/>
-      <c r="T5" s="141"/>
-      <c r="U5" s="141"/>
-      <c r="V5" s="141"/>
-      <c r="W5" s="141"/>
-      <c r="X5" s="141"/>
-      <c r="Y5" s="141"/>
-      <c r="Z5" s="141"/>
-      <c r="AA5" s="141"/>
-      <c r="AB5" s="141"/>
-      <c r="AC5" s="141"/>
-      <c r="AD5" s="141"/>
-      <c r="AE5" s="142"/>
+      <c r="B5" s="150"/>
+      <c r="C5" s="150"/>
+      <c r="D5" s="150"/>
+      <c r="E5" s="150"/>
+      <c r="F5" s="150"/>
+      <c r="G5" s="150"/>
+      <c r="H5" s="150"/>
+      <c r="I5" s="150"/>
+      <c r="J5" s="150"/>
+      <c r="K5" s="150"/>
+      <c r="L5" s="150"/>
+      <c r="M5" s="150"/>
+      <c r="N5" s="150"/>
+      <c r="O5" s="150"/>
+      <c r="P5" s="150"/>
+      <c r="Q5" s="150"/>
+      <c r="R5" s="150"/>
+      <c r="S5" s="150"/>
+      <c r="T5" s="150"/>
+      <c r="U5" s="150"/>
+      <c r="V5" s="150"/>
+      <c r="W5" s="150"/>
+      <c r="X5" s="150"/>
+      <c r="Y5" s="150"/>
+      <c r="Z5" s="150"/>
+      <c r="AA5" s="150"/>
+      <c r="AB5" s="150"/>
+      <c r="AC5" s="150"/>
+      <c r="AD5" s="150"/>
+      <c r="AE5" s="192"/>
     </row>
     <row r="6" spans="1:31" ht="7.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="74"/>
@@ -4304,49 +4019,49 @@
     </row>
     <row r="7" spans="1:31" ht="25.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="74"/>
-      <c r="B7" s="154" t="s">
+      <c r="B7" s="159" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="154"/>
-      <c r="D7" s="154"/>
-      <c r="E7" s="154"/>
-      <c r="F7" s="154"/>
-      <c r="G7" s="155"/>
-      <c r="H7" s="172" t="s">
+      <c r="C7" s="159"/>
+      <c r="D7" s="159"/>
+      <c r="E7" s="159"/>
+      <c r="F7" s="159"/>
+      <c r="G7" s="160"/>
+      <c r="H7" s="136" t="s">
         <v>17</v>
       </c>
-      <c r="I7" s="173"/>
-      <c r="J7" s="174"/>
+      <c r="I7" s="137"/>
+      <c r="J7" s="138"/>
       <c r="K7" s="119" t="s">
         <v>18</v>
       </c>
-      <c r="L7" s="172">
+      <c r="L7" s="136">
         <v>20508972734</v>
       </c>
-      <c r="M7" s="173"/>
-      <c r="N7" s="174"/>
-      <c r="O7" s="153" t="s">
+      <c r="M7" s="137"/>
+      <c r="N7" s="138"/>
+      <c r="O7" s="198" t="s">
         <v>19</v>
       </c>
-      <c r="P7" s="154"/>
-      <c r="Q7" s="155"/>
-      <c r="R7" s="150" t="s">
+      <c r="P7" s="159"/>
+      <c r="Q7" s="160"/>
+      <c r="R7" s="195" t="s">
         <v>20</v>
       </c>
-      <c r="S7" s="151"/>
-      <c r="T7" s="151"/>
-      <c r="U7" s="151"/>
-      <c r="V7" s="152"/>
+      <c r="S7" s="196"/>
+      <c r="T7" s="196"/>
+      <c r="U7" s="196"/>
+      <c r="V7" s="197"/>
       <c r="W7" s="77"/>
       <c r="X7" s="120" t="s">
         <v>21</v>
       </c>
-      <c r="Y7" s="150"/>
-      <c r="Z7" s="151"/>
-      <c r="AA7" s="151"/>
-      <c r="AB7" s="151"/>
-      <c r="AC7" s="151"/>
-      <c r="AD7" s="152"/>
+      <c r="Y7" s="195"/>
+      <c r="Z7" s="196"/>
+      <c r="AA7" s="196"/>
+      <c r="AB7" s="196"/>
+      <c r="AC7" s="196"/>
+      <c r="AD7" s="197"/>
       <c r="AE7" s="78"/>
     </row>
     <row r="8" spans="1:31" ht="7.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -4415,39 +4130,39 @@
       <c r="AE9" s="86"/>
     </row>
     <row r="10" spans="1:31" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="140" t="s">
+      <c r="A10" s="149" t="s">
         <v>22</v>
       </c>
-      <c r="B10" s="141"/>
-      <c r="C10" s="141"/>
-      <c r="D10" s="141"/>
-      <c r="E10" s="141"/>
-      <c r="F10" s="141"/>
-      <c r="G10" s="141"/>
-      <c r="H10" s="141"/>
-      <c r="I10" s="141"/>
-      <c r="J10" s="141"/>
-      <c r="K10" s="141"/>
-      <c r="L10" s="141"/>
-      <c r="M10" s="141"/>
-      <c r="N10" s="141"/>
-      <c r="O10" s="141"/>
-      <c r="P10" s="141"/>
-      <c r="Q10" s="141"/>
-      <c r="R10" s="141"/>
-      <c r="S10" s="141"/>
-      <c r="T10" s="141"/>
-      <c r="U10" s="141"/>
-      <c r="V10" s="141"/>
-      <c r="W10" s="141"/>
-      <c r="X10" s="141"/>
-      <c r="Y10" s="141"/>
-      <c r="Z10" s="141"/>
-      <c r="AA10" s="141"/>
-      <c r="AB10" s="141"/>
-      <c r="AC10" s="141"/>
-      <c r="AD10" s="141"/>
-      <c r="AE10" s="142"/>
+      <c r="B10" s="150"/>
+      <c r="C10" s="150"/>
+      <c r="D10" s="150"/>
+      <c r="E10" s="150"/>
+      <c r="F10" s="150"/>
+      <c r="G10" s="150"/>
+      <c r="H10" s="150"/>
+      <c r="I10" s="150"/>
+      <c r="J10" s="150"/>
+      <c r="K10" s="150"/>
+      <c r="L10" s="150"/>
+      <c r="M10" s="150"/>
+      <c r="N10" s="150"/>
+      <c r="O10" s="150"/>
+      <c r="P10" s="150"/>
+      <c r="Q10" s="150"/>
+      <c r="R10" s="150"/>
+      <c r="S10" s="150"/>
+      <c r="T10" s="150"/>
+      <c r="U10" s="150"/>
+      <c r="V10" s="150"/>
+      <c r="W10" s="150"/>
+      <c r="X10" s="150"/>
+      <c r="Y10" s="150"/>
+      <c r="Z10" s="150"/>
+      <c r="AA10" s="150"/>
+      <c r="AB10" s="150"/>
+      <c r="AC10" s="150"/>
+      <c r="AD10" s="150"/>
+      <c r="AE10" s="192"/>
     </row>
     <row r="11" spans="1:31" ht="7.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="87"/>
@@ -4481,41 +4196,41 @@
     </row>
     <row r="12" spans="1:31" ht="37.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="74"/>
-      <c r="B12" s="143" t="s">
+      <c r="B12" s="151" t="s">
         <v>288</v>
       </c>
-      <c r="C12" s="143"/>
-      <c r="D12" s="143"/>
-      <c r="E12" s="143"/>
-      <c r="F12" s="143"/>
-      <c r="G12" s="144"/>
-      <c r="H12" s="200"/>
-      <c r="I12" s="202"/>
-      <c r="J12" s="202"/>
-      <c r="K12" s="202"/>
-      <c r="L12" s="201"/>
-      <c r="M12" s="185" t="s">
+      <c r="C12" s="151"/>
+      <c r="D12" s="151"/>
+      <c r="E12" s="151"/>
+      <c r="F12" s="151"/>
+      <c r="G12" s="152"/>
+      <c r="H12" s="164"/>
+      <c r="I12" s="169"/>
+      <c r="J12" s="169"/>
+      <c r="K12" s="169"/>
+      <c r="L12" s="165"/>
+      <c r="M12" s="171" t="s">
         <v>289</v>
       </c>
-      <c r="N12" s="186"/>
-      <c r="O12" s="187"/>
-      <c r="P12" s="145"/>
-      <c r="Q12" s="146"/>
-      <c r="R12" s="146"/>
-      <c r="S12" s="146"/>
-      <c r="T12" s="147"/>
-      <c r="U12" s="193" t="s">
+      <c r="N12" s="168"/>
+      <c r="O12" s="172"/>
+      <c r="P12" s="161"/>
+      <c r="Q12" s="162"/>
+      <c r="R12" s="162"/>
+      <c r="S12" s="162"/>
+      <c r="T12" s="163"/>
+      <c r="U12" s="189" t="s">
         <v>211</v>
       </c>
-      <c r="V12" s="194"/>
-      <c r="W12" s="194"/>
-      <c r="X12" s="195"/>
-      <c r="Y12" s="182"/>
-      <c r="Z12" s="183"/>
-      <c r="AA12" s="183"/>
-      <c r="AB12" s="183"/>
-      <c r="AC12" s="183"/>
-      <c r="AD12" s="184"/>
+      <c r="V12" s="190"/>
+      <c r="W12" s="190"/>
+      <c r="X12" s="191"/>
+      <c r="Y12" s="166"/>
+      <c r="Z12" s="170"/>
+      <c r="AA12" s="170"/>
+      <c r="AB12" s="170"/>
+      <c r="AC12" s="170"/>
+      <c r="AD12" s="167"/>
       <c r="AE12" s="90"/>
     </row>
     <row r="13" spans="1:31" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.2">
@@ -4553,43 +4268,43 @@
     </row>
     <row r="14" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A14" s="74"/>
-      <c r="B14" s="143" t="s">
+      <c r="B14" s="151" t="s">
         <v>23</v>
       </c>
-      <c r="C14" s="143"/>
-      <c r="D14" s="143"/>
-      <c r="E14" s="143"/>
-      <c r="F14" s="143"/>
-      <c r="G14" s="144"/>
-      <c r="H14" s="182"/>
-      <c r="I14" s="183"/>
-      <c r="J14" s="183"/>
-      <c r="K14" s="183"/>
-      <c r="L14" s="184"/>
+      <c r="C14" s="151"/>
+      <c r="D14" s="151"/>
+      <c r="E14" s="151"/>
+      <c r="F14" s="151"/>
+      <c r="G14" s="152"/>
+      <c r="H14" s="166"/>
+      <c r="I14" s="170"/>
+      <c r="J14" s="170"/>
+      <c r="K14" s="170"/>
+      <c r="L14" s="167"/>
       <c r="M14" s="86"/>
       <c r="N14" s="86"/>
       <c r="O14" s="85" t="s">
         <v>24</v>
       </c>
-      <c r="P14" s="200"/>
-      <c r="Q14" s="201"/>
+      <c r="P14" s="164"/>
+      <c r="Q14" s="165"/>
       <c r="R14" s="122" t="s">
         <v>25</v>
       </c>
-      <c r="S14" s="182"/>
-      <c r="T14" s="184"/>
+      <c r="S14" s="166"/>
+      <c r="T14" s="167"/>
       <c r="U14" s="121"/>
-      <c r="V14" s="186" t="s">
+      <c r="V14" s="168" t="s">
         <v>14</v>
       </c>
-      <c r="W14" s="186"/>
-      <c r="X14" s="186"/>
-      <c r="Y14" s="206"/>
-      <c r="Z14" s="206"/>
-      <c r="AA14" s="206"/>
-      <c r="AB14" s="206"/>
-      <c r="AC14" s="206"/>
-      <c r="AD14" s="206"/>
+      <c r="W14" s="168"/>
+      <c r="X14" s="168"/>
+      <c r="Y14" s="208"/>
+      <c r="Z14" s="208"/>
+      <c r="AA14" s="208"/>
+      <c r="AB14" s="208"/>
+      <c r="AC14" s="208"/>
+      <c r="AD14" s="208"/>
       <c r="AE14" s="95"/>
     </row>
     <row r="15" spans="1:31" x14ac:dyDescent="0.2">
@@ -4627,38 +4342,38 @@
     </row>
     <row r="16" spans="1:31" ht="46.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="74"/>
-      <c r="B16" s="143" t="s">
+      <c r="B16" s="151" t="s">
         <v>287</v>
       </c>
-      <c r="C16" s="143"/>
-      <c r="D16" s="143"/>
-      <c r="E16" s="143"/>
-      <c r="F16" s="143"/>
-      <c r="G16" s="144"/>
-      <c r="H16" s="203"/>
-      <c r="I16" s="203"/>
-      <c r="J16" s="203"/>
-      <c r="K16" s="203"/>
-      <c r="L16" s="203"/>
-      <c r="M16" s="203"/>
-      <c r="N16" s="203"/>
-      <c r="O16" s="203"/>
-      <c r="P16" s="203"/>
-      <c r="Q16" s="203"/>
-      <c r="R16" s="203"/>
+      <c r="C16" s="151"/>
+      <c r="D16" s="151"/>
+      <c r="E16" s="151"/>
+      <c r="F16" s="151"/>
+      <c r="G16" s="152"/>
+      <c r="H16" s="184"/>
+      <c r="I16" s="184"/>
+      <c r="J16" s="184"/>
+      <c r="K16" s="184"/>
+      <c r="L16" s="184"/>
+      <c r="M16" s="184"/>
+      <c r="N16" s="184"/>
+      <c r="O16" s="184"/>
+      <c r="P16" s="184"/>
+      <c r="Q16" s="184"/>
+      <c r="R16" s="184"/>
       <c r="S16" s="96"/>
-      <c r="T16" s="204" t="s">
+      <c r="T16" s="210" t="s">
         <v>286</v>
       </c>
-      <c r="U16" s="204"/>
-      <c r="V16" s="204"/>
-      <c r="W16" s="204"/>
-      <c r="X16" s="205"/>
-      <c r="Y16" s="207"/>
-      <c r="Z16" s="208"/>
-      <c r="AA16" s="208"/>
-      <c r="AB16" s="208"/>
-      <c r="AC16" s="208"/>
+      <c r="U16" s="210"/>
+      <c r="V16" s="210"/>
+      <c r="W16" s="210"/>
+      <c r="X16" s="211"/>
+      <c r="Y16" s="187"/>
+      <c r="Z16" s="188"/>
+      <c r="AA16" s="188"/>
+      <c r="AB16" s="188"/>
+      <c r="AC16" s="188"/>
       <c r="AD16" s="209"/>
       <c r="AE16" s="97"/>
     </row>
@@ -4697,38 +4412,38 @@
     </row>
     <row r="18" spans="1:31" ht="48.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="74"/>
-      <c r="B18" s="143" t="s">
+      <c r="B18" s="151" t="s">
         <v>13</v>
       </c>
-      <c r="C18" s="143"/>
-      <c r="D18" s="143"/>
-      <c r="E18" s="143"/>
-      <c r="F18" s="143"/>
-      <c r="G18" s="144"/>
-      <c r="H18" s="188"/>
-      <c r="I18" s="188"/>
-      <c r="J18" s="188"/>
-      <c r="K18" s="188"/>
-      <c r="L18" s="188"/>
-      <c r="M18" s="188"/>
-      <c r="N18" s="188"/>
-      <c r="O18" s="188"/>
-      <c r="P18" s="188"/>
-      <c r="Q18" s="188"/>
-      <c r="R18" s="188"/>
-      <c r="T18" s="186" t="s">
+      <c r="C18" s="151"/>
+      <c r="D18" s="151"/>
+      <c r="E18" s="151"/>
+      <c r="F18" s="151"/>
+      <c r="G18" s="152"/>
+      <c r="H18" s="153"/>
+      <c r="I18" s="153"/>
+      <c r="J18" s="153"/>
+      <c r="K18" s="153"/>
+      <c r="L18" s="153"/>
+      <c r="M18" s="153"/>
+      <c r="N18" s="153"/>
+      <c r="O18" s="153"/>
+      <c r="P18" s="153"/>
+      <c r="Q18" s="153"/>
+      <c r="R18" s="153"/>
+      <c r="T18" s="168" t="s">
         <v>27</v>
       </c>
-      <c r="U18" s="186"/>
-      <c r="V18" s="186"/>
-      <c r="W18" s="186"/>
-      <c r="X18" s="187"/>
-      <c r="Y18" s="145"/>
-      <c r="Z18" s="146"/>
-      <c r="AA18" s="146"/>
-      <c r="AB18" s="146"/>
-      <c r="AC18" s="146"/>
-      <c r="AD18" s="147"/>
+      <c r="U18" s="168"/>
+      <c r="V18" s="168"/>
+      <c r="W18" s="168"/>
+      <c r="X18" s="172"/>
+      <c r="Y18" s="161"/>
+      <c r="Z18" s="162"/>
+      <c r="AA18" s="162"/>
+      <c r="AB18" s="162"/>
+      <c r="AC18" s="162"/>
+      <c r="AD18" s="163"/>
       <c r="AE18" s="98"/>
     </row>
     <row r="19" spans="1:31" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.2">
@@ -4766,37 +4481,37 @@
     </row>
     <row r="20" spans="1:31" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="74"/>
-      <c r="B20" s="143" t="s">
+      <c r="B20" s="151" t="s">
         <v>28</v>
       </c>
-      <c r="C20" s="143"/>
-      <c r="D20" s="143"/>
-      <c r="E20" s="143"/>
-      <c r="F20" s="143"/>
-      <c r="G20" s="144"/>
-      <c r="H20" s="145"/>
-      <c r="I20" s="146"/>
-      <c r="J20" s="146"/>
-      <c r="K20" s="146"/>
-      <c r="L20" s="146"/>
-      <c r="M20" s="146"/>
-      <c r="N20" s="146"/>
-      <c r="O20" s="146"/>
-      <c r="P20" s="146"/>
-      <c r="Q20" s="146"/>
-      <c r="R20" s="146"/>
-      <c r="S20" s="146"/>
-      <c r="T20" s="146"/>
-      <c r="U20" s="146"/>
-      <c r="V20" s="146"/>
-      <c r="W20" s="146"/>
-      <c r="X20" s="146"/>
-      <c r="Y20" s="146"/>
-      <c r="Z20" s="146"/>
-      <c r="AA20" s="146"/>
-      <c r="AB20" s="146"/>
-      <c r="AC20" s="146"/>
-      <c r="AD20" s="147"/>
+      <c r="C20" s="151"/>
+      <c r="D20" s="151"/>
+      <c r="E20" s="151"/>
+      <c r="F20" s="151"/>
+      <c r="G20" s="152"/>
+      <c r="H20" s="141"/>
+      <c r="I20" s="142"/>
+      <c r="J20" s="142"/>
+      <c r="K20" s="142"/>
+      <c r="L20" s="142"/>
+      <c r="M20" s="142"/>
+      <c r="N20" s="142"/>
+      <c r="O20" s="142"/>
+      <c r="P20" s="142"/>
+      <c r="Q20" s="142"/>
+      <c r="R20" s="142"/>
+      <c r="S20" s="142"/>
+      <c r="T20" s="142"/>
+      <c r="U20" s="142"/>
+      <c r="V20" s="142"/>
+      <c r="W20" s="142"/>
+      <c r="X20" s="142"/>
+      <c r="Y20" s="142"/>
+      <c r="Z20" s="142"/>
+      <c r="AA20" s="142"/>
+      <c r="AB20" s="142"/>
+      <c r="AC20" s="142"/>
+      <c r="AD20" s="143"/>
       <c r="AE20" s="99"/>
     </row>
     <row r="21" spans="1:31" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.2">
@@ -4834,27 +4549,27 @@
     </row>
     <row r="22" spans="1:31" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="74"/>
-      <c r="B22" s="143" t="s">
+      <c r="B22" s="151" t="s">
         <v>283</v>
       </c>
-      <c r="C22" s="143"/>
-      <c r="D22" s="143"/>
-      <c r="E22" s="143"/>
-      <c r="F22" s="143"/>
-      <c r="G22" s="144"/>
-      <c r="H22" s="188" t="s">
+      <c r="C22" s="151"/>
+      <c r="D22" s="151"/>
+      <c r="E22" s="151"/>
+      <c r="F22" s="151"/>
+      <c r="G22" s="152"/>
+      <c r="H22" s="153" t="s">
         <v>290</v>
       </c>
-      <c r="I22" s="188"/>
-      <c r="J22" s="188"/>
-      <c r="K22" s="188"/>
-      <c r="L22" s="188"/>
-      <c r="M22" s="188"/>
-      <c r="N22" s="188"/>
-      <c r="O22" s="188"/>
-      <c r="P22" s="188"/>
-      <c r="Q22" s="188"/>
-      <c r="R22" s="188"/>
+      <c r="I22" s="153"/>
+      <c r="J22" s="153"/>
+      <c r="K22" s="153"/>
+      <c r="L22" s="153"/>
+      <c r="M22" s="153"/>
+      <c r="N22" s="153"/>
+      <c r="O22" s="153"/>
+      <c r="P22" s="153"/>
+      <c r="Q22" s="153"/>
+      <c r="R22" s="153"/>
       <c r="S22" s="127"/>
       <c r="T22" s="127"/>
       <c r="U22" s="127"/>
@@ -4862,13 +4577,13 @@
       <c r="W22" s="85" t="s">
         <v>291</v>
       </c>
-      <c r="X22" s="188"/>
-      <c r="Y22" s="188"/>
-      <c r="Z22" s="188"/>
-      <c r="AA22" s="188"/>
-      <c r="AB22" s="188"/>
-      <c r="AC22" s="188"/>
-      <c r="AD22" s="188"/>
+      <c r="X22" s="154"/>
+      <c r="Y22" s="154"/>
+      <c r="Z22" s="154"/>
+      <c r="AA22" s="154"/>
+      <c r="AB22" s="154"/>
+      <c r="AC22" s="154"/>
+      <c r="AD22" s="154"/>
       <c r="AE22" s="99"/>
     </row>
     <row r="23" spans="1:31" ht="7.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -4907,43 +4622,43 @@
     <row r="24" spans="1:31" ht="13.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D24" s="117"/>
       <c r="E24" s="117"/>
-      <c r="F24" s="146"/>
-      <c r="G24" s="146"/>
-      <c r="H24" s="146"/>
-      <c r="I24" s="146"/>
-      <c r="J24" s="146"/>
-      <c r="K24" s="146"/>
-      <c r="L24" s="146"/>
-      <c r="M24" s="146"/>
-      <c r="N24" s="146"/>
-      <c r="O24" s="146"/>
-      <c r="P24" s="146"/>
-      <c r="Q24" s="146"/>
-      <c r="R24" s="146"/>
-      <c r="S24" s="146"/>
-      <c r="T24" s="146"/>
-      <c r="U24" s="146"/>
-      <c r="V24" s="146"/>
-      <c r="W24" s="146"/>
-      <c r="X24" s="146"/>
-      <c r="Y24" s="146"/>
-      <c r="Z24" s="146"/>
-      <c r="AA24" s="146"/>
-      <c r="AB24" s="146"/>
-      <c r="AC24" s="146"/>
-      <c r="AD24" s="146"/>
-      <c r="AE24" s="146"/>
+      <c r="F24" s="162"/>
+      <c r="G24" s="162"/>
+      <c r="H24" s="162"/>
+      <c r="I24" s="162"/>
+      <c r="J24" s="162"/>
+      <c r="K24" s="162"/>
+      <c r="L24" s="162"/>
+      <c r="M24" s="162"/>
+      <c r="N24" s="162"/>
+      <c r="O24" s="162"/>
+      <c r="P24" s="162"/>
+      <c r="Q24" s="162"/>
+      <c r="R24" s="162"/>
+      <c r="S24" s="162"/>
+      <c r="T24" s="162"/>
+      <c r="U24" s="162"/>
+      <c r="V24" s="162"/>
+      <c r="W24" s="162"/>
+      <c r="X24" s="162"/>
+      <c r="Y24" s="162"/>
+      <c r="Z24" s="162"/>
+      <c r="AA24" s="162"/>
+      <c r="AB24" s="162"/>
+      <c r="AC24" s="162"/>
+      <c r="AD24" s="162"/>
+      <c r="AE24" s="162"/>
     </row>
     <row r="25" spans="1:31" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="140" t="s">
+      <c r="A25" s="149" t="s">
         <v>30</v>
       </c>
-      <c r="B25" s="141"/>
-      <c r="C25" s="141"/>
-      <c r="D25" s="141"/>
-      <c r="E25" s="141"/>
-      <c r="F25" s="141"/>
-      <c r="G25" s="141"/>
+      <c r="B25" s="150"/>
+      <c r="C25" s="150"/>
+      <c r="D25" s="150"/>
+      <c r="E25" s="150"/>
+      <c r="F25" s="150"/>
+      <c r="G25" s="150"/>
       <c r="H25" s="103"/>
       <c r="I25" s="103"/>
       <c r="J25" s="103"/>
@@ -4970,96 +4685,96 @@
       <c r="AE25" s="104"/>
     </row>
     <row r="26" spans="1:31" ht="3.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="178"/>
-      <c r="B26" s="179"/>
-      <c r="C26" s="179"/>
-      <c r="D26" s="179"/>
-      <c r="E26" s="179"/>
-      <c r="F26" s="179"/>
-      <c r="G26" s="179"/>
-      <c r="H26" s="179"/>
-      <c r="I26" s="179"/>
-      <c r="J26" s="179"/>
-      <c r="K26" s="179"/>
-      <c r="L26" s="179"/>
-      <c r="M26" s="179"/>
-      <c r="N26" s="179"/>
-      <c r="O26" s="179"/>
-      <c r="P26" s="179"/>
-      <c r="Q26" s="179"/>
-      <c r="R26" s="179"/>
-      <c r="S26" s="179"/>
-      <c r="T26" s="179"/>
-      <c r="U26" s="179"/>
-      <c r="V26" s="179"/>
-      <c r="W26" s="179"/>
-      <c r="X26" s="179"/>
-      <c r="Y26" s="179"/>
-      <c r="Z26" s="179"/>
-      <c r="AA26" s="179"/>
-      <c r="AB26" s="179"/>
-      <c r="AC26" s="179"/>
-      <c r="AD26" s="179"/>
-      <c r="AE26" s="180"/>
+      <c r="A26" s="145"/>
+      <c r="B26" s="146"/>
+      <c r="C26" s="146"/>
+      <c r="D26" s="146"/>
+      <c r="E26" s="146"/>
+      <c r="F26" s="146"/>
+      <c r="G26" s="146"/>
+      <c r="H26" s="146"/>
+      <c r="I26" s="146"/>
+      <c r="J26" s="146"/>
+      <c r="K26" s="146"/>
+      <c r="L26" s="146"/>
+      <c r="M26" s="146"/>
+      <c r="N26" s="146"/>
+      <c r="O26" s="146"/>
+      <c r="P26" s="146"/>
+      <c r="Q26" s="146"/>
+      <c r="R26" s="146"/>
+      <c r="S26" s="146"/>
+      <c r="T26" s="146"/>
+      <c r="U26" s="146"/>
+      <c r="V26" s="146"/>
+      <c r="W26" s="146"/>
+      <c r="X26" s="146"/>
+      <c r="Y26" s="146"/>
+      <c r="Z26" s="146"/>
+      <c r="AA26" s="146"/>
+      <c r="AB26" s="146"/>
+      <c r="AC26" s="146"/>
+      <c r="AD26" s="146"/>
+      <c r="AE26" s="147"/>
     </row>
     <row r="27" spans="1:31" ht="52.9" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="175" t="s">
+      <c r="A27" s="139" t="s">
         <v>1</v>
       </c>
-      <c r="B27" s="176"/>
+      <c r="B27" s="140"/>
       <c r="C27" s="105" t="s">
         <v>8</v>
       </c>
-      <c r="D27" s="175" t="s">
+      <c r="D27" s="139" t="s">
         <v>9</v>
       </c>
-      <c r="E27" s="181"/>
-      <c r="F27" s="181"/>
-      <c r="G27" s="181"/>
-      <c r="H27" s="181"/>
-      <c r="I27" s="176"/>
-      <c r="J27" s="175" t="s">
+      <c r="E27" s="148"/>
+      <c r="F27" s="148"/>
+      <c r="G27" s="148"/>
+      <c r="H27" s="148"/>
+      <c r="I27" s="140"/>
+      <c r="J27" s="139" t="s">
         <v>10</v>
       </c>
-      <c r="K27" s="181"/>
-      <c r="L27" s="175" t="s">
+      <c r="K27" s="148"/>
+      <c r="L27" s="139" t="s">
         <v>29</v>
       </c>
-      <c r="M27" s="181"/>
-      <c r="N27" s="176"/>
-      <c r="O27" s="175" t="s">
+      <c r="M27" s="148"/>
+      <c r="N27" s="140"/>
+      <c r="O27" s="139" t="s">
         <v>285</v>
       </c>
-      <c r="P27" s="181"/>
-      <c r="Q27" s="176"/>
+      <c r="P27" s="148"/>
+      <c r="Q27" s="140"/>
       <c r="R27" s="105" t="s">
         <v>2</v>
       </c>
-      <c r="S27" s="175" t="s">
+      <c r="S27" s="139" t="s">
         <v>284</v>
       </c>
-      <c r="T27" s="181"/>
-      <c r="U27" s="181"/>
-      <c r="V27" s="181"/>
+      <c r="T27" s="148"/>
+      <c r="U27" s="148"/>
+      <c r="V27" s="148"/>
       <c r="W27" s="105" t="s">
         <v>11</v>
       </c>
       <c r="X27" s="105" t="s">
         <v>3</v>
       </c>
-      <c r="Y27" s="175" t="s">
+      <c r="Y27" s="139" t="s">
         <v>12</v>
       </c>
-      <c r="Z27" s="181"/>
-      <c r="AA27" s="181"/>
-      <c r="AB27" s="176"/>
+      <c r="Z27" s="148"/>
+      <c r="AA27" s="148"/>
+      <c r="AB27" s="140"/>
       <c r="AC27" s="128" t="s">
         <v>31</v>
       </c>
-      <c r="AD27" s="177" t="s">
+      <c r="AD27" s="144" t="s">
         <v>292</v>
       </c>
-      <c r="AE27" s="177"/>
+      <c r="AE27" s="144"/>
     </row>
     <row r="28" spans="1:31" ht="13.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="116"/>
@@ -7230,6 +6945,7 @@
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" selectLockedCells="1" sort="0" autoFilter="0" pivotTables="0"/>
   <mergeCells count="57">
+    <mergeCell ref="AB1:AE3"/>
     <mergeCell ref="AB14:AD14"/>
     <mergeCell ref="Y16:AD16"/>
     <mergeCell ref="Y27:AB27"/>
@@ -7237,16 +6953,23 @@
     <mergeCell ref="T18:X18"/>
     <mergeCell ref="S27:V27"/>
     <mergeCell ref="Y14:AA14"/>
+    <mergeCell ref="F24:AE24"/>
+    <mergeCell ref="A1:G3"/>
     <mergeCell ref="H18:R18"/>
     <mergeCell ref="H16:R16"/>
     <mergeCell ref="R2:V2"/>
     <mergeCell ref="B20:G20"/>
     <mergeCell ref="B18:G18"/>
-    <mergeCell ref="F24:AE24"/>
     <mergeCell ref="P2:Q2"/>
     <mergeCell ref="U12:X12"/>
-    <mergeCell ref="Y3:AA3"/>
-    <mergeCell ref="W3:X3"/>
+    <mergeCell ref="A5:AE5"/>
+    <mergeCell ref="A10:AE10"/>
+    <mergeCell ref="B16:G16"/>
+    <mergeCell ref="P12:T12"/>
+    <mergeCell ref="X2:AA2"/>
+    <mergeCell ref="Y7:AD7"/>
+    <mergeCell ref="R7:V7"/>
+    <mergeCell ref="O7:Q7"/>
     <mergeCell ref="B7:G7"/>
     <mergeCell ref="Y18:AD18"/>
     <mergeCell ref="P14:Q14"/>
@@ -7256,37 +6979,29 @@
     <mergeCell ref="H12:L12"/>
     <mergeCell ref="H14:L14"/>
     <mergeCell ref="H7:J7"/>
+    <mergeCell ref="B14:G14"/>
+    <mergeCell ref="Y12:AD12"/>
+    <mergeCell ref="M12:O12"/>
     <mergeCell ref="A27:B27"/>
     <mergeCell ref="H20:AD20"/>
     <mergeCell ref="AD27:AE27"/>
     <mergeCell ref="A26:AE26"/>
     <mergeCell ref="D27:I27"/>
     <mergeCell ref="A25:G25"/>
-    <mergeCell ref="B14:G14"/>
     <mergeCell ref="B22:G22"/>
     <mergeCell ref="J27:K27"/>
     <mergeCell ref="L27:N27"/>
-    <mergeCell ref="Y12:AD12"/>
-    <mergeCell ref="M12:O12"/>
     <mergeCell ref="H22:R22"/>
     <mergeCell ref="X22:AD22"/>
     <mergeCell ref="O27:Q27"/>
-    <mergeCell ref="R3:V3"/>
-    <mergeCell ref="A1:G3"/>
-    <mergeCell ref="A5:AE5"/>
-    <mergeCell ref="A10:AE10"/>
-    <mergeCell ref="B16:G16"/>
-    <mergeCell ref="P12:T12"/>
-    <mergeCell ref="X2:AA2"/>
-    <mergeCell ref="Y7:AD7"/>
-    <mergeCell ref="R7:V7"/>
-    <mergeCell ref="O7:Q7"/>
-    <mergeCell ref="AB1:AE3"/>
     <mergeCell ref="H1:AA1"/>
     <mergeCell ref="I2:O2"/>
     <mergeCell ref="I3:O3"/>
     <mergeCell ref="P3:Q3"/>
     <mergeCell ref="L7:N7"/>
+    <mergeCell ref="Y3:AA3"/>
+    <mergeCell ref="W3:X3"/>
+    <mergeCell ref="R3:V3"/>
   </mergeCells>
   <printOptions horizontalCentered="1" gridLinesSet="0"/>
   <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.19685039370078741" bottom="0.35433070866141736" header="0.11811023622047245" footer="0.19685039370078741"/>
@@ -7298,10 +7013,9 @@
     <ignoredError sqref="X2" numberStoredAsText="1"/>
   </ignoredErrors>
   <drawing r:id="rId2"/>
-  <legacyDrawing r:id="rId3"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" disablePrompts="1" count="3">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000001000000}">
           <x14:formula1>
             <xm:f>Datos!$B$3:$D$3</xm:f>
@@ -7337,14 +7051,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="210" t="s">
+      <c r="A1" s="212" t="s">
         <v>115</v>
       </c>
-      <c r="B1" s="211"/>
-      <c r="D1" s="210" t="s">
+      <c r="B1" s="213"/>
+      <c r="D1" s="212" t="s">
         <v>116</v>
       </c>
-      <c r="E1" s="211"/>
+      <c r="E1" s="213"/>
     </row>
     <row r="2" spans="1:5" s="4" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
@@ -8162,20 +7876,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="215" t="s">
+      <c r="A1" s="217" t="s">
         <v>115</v>
       </c>
-      <c r="B1" s="216"/>
-      <c r="C1" s="216"/>
-      <c r="D1" s="217"/>
+      <c r="B1" s="218"/>
+      <c r="C1" s="218"/>
+      <c r="D1" s="219"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" s="212" t="s">
+      <c r="A2" s="214" t="s">
         <v>194</v>
       </c>
-      <c r="B2" s="213"/>
-      <c r="C2" s="213"/>
-      <c r="D2" s="214"/>
+      <c r="B2" s="215"/>
+      <c r="C2" s="215"/>
+      <c r="D2" s="216"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="34" t="s">
@@ -8242,12 +7956,12 @@
       <c r="D7" s="48"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A8" s="212" t="s">
+      <c r="A8" s="214" t="s">
         <v>203</v>
       </c>
-      <c r="B8" s="213"/>
-      <c r="C8" s="213"/>
-      <c r="D8" s="214"/>
+      <c r="B8" s="215"/>
+      <c r="C8" s="215"/>
+      <c r="D8" s="216"/>
     </row>
     <row r="9" spans="1:8" ht="23.65" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="34" t="s">
@@ -8312,12 +8026,12 @@
       <c r="H13" s="33"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A14" s="212" t="s">
+      <c r="A14" s="214" t="s">
         <v>208</v>
       </c>
-      <c r="B14" s="213"/>
-      <c r="C14" s="213"/>
-      <c r="D14" s="214"/>
+      <c r="B14" s="215"/>
+      <c r="C14" s="215"/>
+      <c r="D14" s="216"/>
     </row>
     <row r="15" spans="1:8" ht="15.6" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="45"/>
@@ -8864,10 +8578,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" s="218" t="s">
+      <c r="A1" s="220" t="s">
         <v>123</v>
       </c>
-      <c r="B1" s="218"/>
+      <c r="B1" s="220"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" s="22">
@@ -9292,19 +9006,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A1" s="219" t="s">
+      <c r="A1" s="221" t="s">
         <v>210</v>
       </c>
-      <c r="B1" s="220"/>
-      <c r="C1" s="220"/>
-      <c r="D1" s="220"/>
-      <c r="E1" s="220"/>
-      <c r="F1" s="220"/>
-      <c r="G1" s="220"/>
-      <c r="H1" s="220"/>
-      <c r="I1" s="220"/>
-      <c r="J1" s="220"/>
-      <c r="K1" s="221"/>
+      <c r="B1" s="222"/>
+      <c r="C1" s="222"/>
+      <c r="D1" s="222"/>
+      <c r="E1" s="222"/>
+      <c r="F1" s="222"/>
+      <c r="G1" s="222"/>
+      <c r="H1" s="222"/>
+      <c r="I1" s="222"/>
+      <c r="J1" s="222"/>
+      <c r="K1" s="223"/>
       <c r="N1" s="63"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Cambio de posiciones de inputs y persistencia en filtros de listado
</commit_message>
<xml_diff>
--- a/GestionAmbiental/wwwroot/ExcelTemplates/Inspecciones/JU-MAP-PRO-004.F01_Inspección_V01.xlsx
+++ b/GestionAmbiental/wwwroot/ExcelTemplates/Inspecciones/JU-MAP-PRO-004.F01_Inspección_V01.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Electrodata\Marcobre\Gestiona Marcobre\Marcobre-GestionAmbiental\GestionAmbiental\wwwroot\ExcelTemplates\Inspecciones\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C36B8806-8767-4E17-A45A-0A6D6753CADE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E2576EC-B162-44FF-B18B-5E0520D1C8DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="813" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="3">'Nivel Riesgo MA'!$A$1:$D$39</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="5">'Nivel Riesgo SSO'!$A$1:$K$21</definedName>
   </definedNames>
-  <calcPr calcId="191029" calcOnSave="0" concurrentCalc="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -129,9 +129,6 @@
     <t>Registro N°:</t>
   </si>
   <si>
-    <t>Responsable de la inspección:</t>
-  </si>
-  <si>
     <t xml:space="preserve">Objetivo de la inspección: </t>
   </si>
   <si>
@@ -946,6 +943,9 @@
   </si>
   <si>
     <t>Estado</t>
+  </si>
+  <si>
+    <t>Lider de la inspección:</t>
   </si>
 </sst>
 </file>
@@ -1330,7 +1330,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="0"/>
   </cellStyleXfs>
-  <cellXfs count="224">
+  <cellXfs count="225">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1688,6 +1688,216 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1709,63 +1919,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1778,165 +1931,12 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1972,6 +1972,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="13" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2728,32 +2731,32 @@
   <sheetData>
     <row r="1" spans="1:79" s="10" customFormat="1" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B1" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="C1" s="9" t="s">
         <v>36</v>
-      </c>
-      <c r="C1" s="9" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:79" s="10" customFormat="1" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="D3" s="9" t="s">
         <v>33</v>
-      </c>
-      <c r="B3" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="C3" s="9" t="s">
-        <v>212</v>
-      </c>
-      <c r="D3" s="9" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:79" s="10" customFormat="1" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B5" s="11" t="e">
         <f>IF(Inspección!#REF!="MA","Tolerable","")</f>
@@ -2782,241 +2785,241 @@
     </row>
     <row r="7" spans="1:79" s="16" customFormat="1" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="B7" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="D7" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="E7" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="F7" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="G7" s="14" t="s">
+        <v>44</v>
+      </c>
+      <c r="H7" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="I7" s="14" t="s">
+        <v>46</v>
+      </c>
+      <c r="J7" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="K7" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="L7" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="M7" s="14" t="s">
+        <v>50</v>
+      </c>
+      <c r="N7" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="O7" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="P7" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q7" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="R7" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="S7" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="B7" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="C7" s="14" t="s">
-        <v>41</v>
-      </c>
-      <c r="D7" s="14" t="s">
-        <v>42</v>
-      </c>
-      <c r="E7" s="14" t="s">
-        <v>43</v>
-      </c>
-      <c r="F7" s="14" t="s">
-        <v>44</v>
-      </c>
-      <c r="G7" s="14" t="s">
-        <v>45</v>
-      </c>
-      <c r="H7" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="I7" s="14" t="s">
-        <v>47</v>
-      </c>
-      <c r="J7" s="14" t="s">
-        <v>48</v>
-      </c>
-      <c r="K7" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="L7" s="14" t="s">
-        <v>50</v>
-      </c>
-      <c r="M7" s="14" t="s">
-        <v>51</v>
-      </c>
-      <c r="N7" s="14" t="s">
-        <v>52</v>
-      </c>
-      <c r="O7" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="P7" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="Q7" s="14" t="s">
+      <c r="T7" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="R7" s="14" t="s">
-        <v>119</v>
-      </c>
-      <c r="S7" s="8" t="s">
-        <v>114</v>
-      </c>
-      <c r="T7" s="14" t="s">
+      <c r="U7" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="U7" s="14" t="s">
+      <c r="V7" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="V7" s="14" t="s">
+      <c r="W7" s="14" t="s">
         <v>58</v>
       </c>
-      <c r="W7" s="14" t="s">
+      <c r="X7" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="X7" s="14" t="s">
+      <c r="Y7" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="Y7" s="14" t="s">
+      <c r="Z7" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="Z7" s="14" t="s">
+      <c r="AA7" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="AA7" s="14" t="s">
+      <c r="AB7" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="AB7" s="14" t="s">
+      <c r="AC7" s="14" t="s">
         <v>64</v>
       </c>
-      <c r="AC7" s="14" t="s">
+      <c r="AD7" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="AE7" s="14" t="s">
         <v>65</v>
       </c>
-      <c r="AD7" s="14" t="s">
+      <c r="AF7" s="14" t="s">
         <v>67</v>
       </c>
-      <c r="AE7" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="AF7" s="14" t="s">
+      <c r="AG7" s="14" t="s">
         <v>68</v>
       </c>
-      <c r="AG7" s="14" t="s">
+      <c r="AH7" s="14" t="s">
         <v>69</v>
       </c>
-      <c r="AH7" s="14" t="s">
+      <c r="AI7" s="14" t="s">
         <v>70</v>
       </c>
-      <c r="AI7" s="14" t="s">
+      <c r="AJ7" s="14" t="s">
         <v>71</v>
       </c>
-      <c r="AJ7" s="14" t="s">
+      <c r="AK7" s="14" t="s">
         <v>72</v>
       </c>
-      <c r="AK7" s="14" t="s">
+      <c r="AL7" s="14" t="s">
         <v>73</v>
       </c>
-      <c r="AL7" s="14" t="s">
+      <c r="AM7" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="AM7" s="14" t="s">
+      <c r="AN7" s="14" t="s">
         <v>75</v>
       </c>
-      <c r="AN7" s="14" t="s">
+      <c r="AO7" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="AP7" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="AO7" s="8" t="s">
+      <c r="AQ7" s="15" t="s">
+        <v>77</v>
+      </c>
+      <c r="AR7" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="AS7" s="15" t="s">
+        <v>79</v>
+      </c>
+      <c r="AT7" s="15" t="s">
+        <v>80</v>
+      </c>
+      <c r="AU7" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="AV7" s="15" t="s">
+        <v>82</v>
+      </c>
+      <c r="AW7" s="15" t="s">
+        <v>83</v>
+      </c>
+      <c r="AX7" s="15" t="s">
+        <v>84</v>
+      </c>
+      <c r="AY7" s="15" t="s">
+        <v>85</v>
+      </c>
+      <c r="AZ7" s="15" t="s">
+        <v>86</v>
+      </c>
+      <c r="BA7" s="15" t="s">
+        <v>87</v>
+      </c>
+      <c r="BB7" s="15" t="s">
+        <v>88</v>
+      </c>
+      <c r="BC7" s="15" t="s">
+        <v>89</v>
+      </c>
+      <c r="BD7" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="BE7" s="15" t="s">
+        <v>91</v>
+      </c>
+      <c r="BF7" s="15" t="s">
+        <v>92</v>
+      </c>
+      <c r="BG7" s="15" t="s">
+        <v>93</v>
+      </c>
+      <c r="BH7" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="BI7" s="8" t="s">
         <v>117</v>
       </c>
-      <c r="AP7" s="15" t="s">
-        <v>77</v>
-      </c>
-      <c r="AQ7" s="15" t="s">
-        <v>78</v>
-      </c>
-      <c r="AR7" s="15" t="s">
-        <v>79</v>
-      </c>
-      <c r="AS7" s="15" t="s">
-        <v>80</v>
-      </c>
-      <c r="AT7" s="15" t="s">
-        <v>81</v>
-      </c>
-      <c r="AU7" s="15" t="s">
-        <v>82</v>
-      </c>
-      <c r="AV7" s="15" t="s">
-        <v>83</v>
-      </c>
-      <c r="AW7" s="15" t="s">
-        <v>84</v>
-      </c>
-      <c r="AX7" s="15" t="s">
-        <v>85</v>
-      </c>
-      <c r="AY7" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="AZ7" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="BA7" s="15" t="s">
-        <v>88</v>
-      </c>
-      <c r="BB7" s="15" t="s">
-        <v>89</v>
-      </c>
-      <c r="BC7" s="15" t="s">
-        <v>90</v>
-      </c>
-      <c r="BD7" s="15" t="s">
-        <v>91</v>
-      </c>
-      <c r="BE7" s="15" t="s">
-        <v>92</v>
-      </c>
-      <c r="BF7" s="15" t="s">
-        <v>93</v>
-      </c>
-      <c r="BG7" s="15" t="s">
+      <c r="BJ7" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="BK7" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="BL7" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="BM7" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="BN7" s="14" t="s">
         <v>94</v>
       </c>
-      <c r="BH7" s="14" t="s">
-        <v>119</v>
-      </c>
-      <c r="BI7" s="8" t="s">
-        <v>118</v>
-      </c>
-      <c r="BJ7" s="14" t="s">
-        <v>112</v>
-      </c>
-      <c r="BK7" s="14" t="s">
-        <v>111</v>
-      </c>
-      <c r="BL7" s="14" t="s">
-        <v>110</v>
-      </c>
-      <c r="BM7" s="14" t="s">
-        <v>109</v>
-      </c>
-      <c r="BN7" s="14" t="s">
+      <c r="BO7" s="14" t="s">
+        <v>107</v>
+      </c>
+      <c r="BP7" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="BQ7" s="14" t="s">
+        <v>105</v>
+      </c>
+      <c r="BR7" s="14" t="s">
+        <v>104</v>
+      </c>
+      <c r="BS7" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="BT7" s="14" t="s">
+        <v>102</v>
+      </c>
+      <c r="BU7" s="14" t="s">
+        <v>101</v>
+      </c>
+      <c r="BV7" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="BW7" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="BX7" s="14" t="s">
+        <v>98</v>
+      </c>
+      <c r="BY7" s="14" t="s">
+        <v>97</v>
+      </c>
+      <c r="BZ7" s="14" t="s">
+        <v>96</v>
+      </c>
+      <c r="CA7" s="14" t="s">
         <v>95</v>
-      </c>
-      <c r="BO7" s="14" t="s">
-        <v>108</v>
-      </c>
-      <c r="BP7" s="14" t="s">
-        <v>107</v>
-      </c>
-      <c r="BQ7" s="14" t="s">
-        <v>106</v>
-      </c>
-      <c r="BR7" s="14" t="s">
-        <v>105</v>
-      </c>
-      <c r="BS7" s="14" t="s">
-        <v>104</v>
-      </c>
-      <c r="BT7" s="14" t="s">
-        <v>103</v>
-      </c>
-      <c r="BU7" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="BV7" s="14" t="s">
-        <v>101</v>
-      </c>
-      <c r="BW7" s="14" t="s">
-        <v>100</v>
-      </c>
-      <c r="BX7" s="14" t="s">
-        <v>99</v>
-      </c>
-      <c r="BY7" s="14" t="s">
-        <v>98</v>
-      </c>
-      <c r="BZ7" s="14" t="s">
-        <v>97</v>
-      </c>
-      <c r="CA7" s="14" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="8" spans="1:79" s="109" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3341,390 +3344,390 @@
     <row r="10" spans="1:79" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="11" spans="1:79" ht="15" x14ac:dyDescent="0.25">
       <c r="A11" s="110" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B11" s="111"/>
       <c r="C11" s="110" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="12" spans="1:79" ht="15" x14ac:dyDescent="0.25">
       <c r="A12" s="112" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B12" s="111"/>
       <c r="C12" s="113" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="13" spans="1:79" ht="15" x14ac:dyDescent="0.25">
       <c r="A13" s="112" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B13" s="111"/>
       <c r="C13" s="113" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="14" spans="1:79" ht="15" x14ac:dyDescent="0.25">
       <c r="A14" s="112" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B14" s="111"/>
       <c r="C14" s="113" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="15" spans="1:79" ht="15" x14ac:dyDescent="0.25">
       <c r="A15" s="112" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B15" s="111"/>
       <c r="C15" s="113" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="16" spans="1:79" ht="15" x14ac:dyDescent="0.25">
       <c r="A16" s="112" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B16" s="111"/>
       <c r="C16" s="113" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A17" s="111" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B17" s="111"/>
       <c r="C17" s="113" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A18" s="111" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B18" s="111"/>
       <c r="C18" s="113" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="15" x14ac:dyDescent="0.2">
       <c r="A19" s="112" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B19" s="114"/>
       <c r="C19" s="113" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A20" s="112" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B20" s="111"/>
       <c r="C20" s="113" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A21" s="112" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B21" s="111"/>
       <c r="C21" s="113" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A22" s="111" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B22" s="111"/>
       <c r="C22" s="113" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A23" s="111" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B23" s="111"/>
       <c r="C23" s="113" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A24" s="112" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B24" s="111"/>
       <c r="C24" s="113" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A25" s="112" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B25" s="111"/>
       <c r="C25" s="113" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A26" s="112" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B26" s="111"/>
       <c r="C26" s="113" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A27" s="112" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B27" s="111"/>
       <c r="C27" s="113" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A28" s="112" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B28" s="111"/>
       <c r="C28" s="113" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A29" s="111" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B29" s="111"/>
       <c r="C29" s="113" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A30" s="111" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B30" s="111"/>
       <c r="C30" s="113" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A31" s="112" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B31" s="111"/>
       <c r="C31" s="111"/>
     </row>
     <row r="32" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A32" s="111" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B32" s="111"/>
       <c r="C32" s="111"/>
     </row>
     <row r="33" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A33" s="112" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B33" s="111"/>
       <c r="C33" s="111"/>
     </row>
     <row r="34" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A34" s="112" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B34" s="111"/>
       <c r="C34" s="111"/>
     </row>
     <row r="35" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A35" s="111" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B35" s="111"/>
       <c r="C35" s="111"/>
     </row>
     <row r="36" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A36" s="111" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B36" s="111"/>
       <c r="C36" s="111"/>
     </row>
     <row r="37" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A37" s="112" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B37" s="111"/>
       <c r="C37" s="111"/>
     </row>
     <row r="38" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A38" s="112" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B38" s="111"/>
       <c r="C38" s="111"/>
     </row>
     <row r="39" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A39" s="115" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B39" s="111"/>
       <c r="C39" s="111"/>
     </row>
     <row r="40" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A40" s="112" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B40" s="111"/>
       <c r="C40" s="111"/>
     </row>
     <row r="41" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A41" s="112" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B41" s="111"/>
       <c r="C41" s="111"/>
     </row>
     <row r="42" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A42" s="112" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B42" s="111"/>
       <c r="C42" s="111"/>
     </row>
     <row r="43" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A43" s="111" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B43" s="111"/>
       <c r="C43" s="111"/>
     </row>
     <row r="44" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A44" s="111" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B44" s="111"/>
       <c r="C44" s="111"/>
     </row>
     <row r="45" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A45" s="112" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B45" s="111"/>
       <c r="C45" s="111"/>
     </row>
     <row r="46" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A46" s="112" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B46" s="111"/>
       <c r="C46" s="111"/>
     </row>
     <row r="47" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A47" s="112" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B47" s="111"/>
       <c r="C47" s="111"/>
     </row>
     <row r="48" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A48" s="112" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B48" s="111"/>
       <c r="C48" s="111"/>
     </row>
     <row r="49" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A49" s="111" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B49" s="111"/>
       <c r="C49" s="111"/>
     </row>
     <row r="50" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A50" s="112" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B50" s="111"/>
       <c r="C50" s="111"/>
     </row>
     <row r="51" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A51" s="111" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B51" s="111"/>
       <c r="C51" s="111"/>
     </row>
     <row r="52" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A52" s="112" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B52" s="111"/>
       <c r="C52" s="111"/>
     </row>
     <row r="53" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A53" s="111" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B53" s="111"/>
       <c r="C53" s="111"/>
     </row>
     <row r="54" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A54" s="112" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B54" s="111"/>
       <c r="C54" s="111"/>
     </row>
     <row r="55" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A55" s="112" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B55" s="111"/>
       <c r="C55" s="111"/>
     </row>
     <row r="56" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A56" s="112" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B56" s="111"/>
       <c r="C56" s="111"/>
     </row>
     <row r="57" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A57" s="111" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B57" s="111"/>
       <c r="C57" s="111"/>
     </row>
     <row r="58" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A58" s="111" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B58" s="111"/>
       <c r="C58" s="111"/>
     </row>
     <row r="59" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A59" s="112" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B59" s="111"/>
       <c r="C59" s="111"/>
     </row>
     <row r="60" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A60" s="111" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B60" s="111"/>
       <c r="C60" s="111"/>
@@ -3797,125 +3800,125 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:31" ht="20.65" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="175"/>
-      <c r="B1" s="176"/>
-      <c r="C1" s="176"/>
-      <c r="D1" s="176"/>
-      <c r="E1" s="176"/>
-      <c r="F1" s="176"/>
-      <c r="G1" s="177"/>
-      <c r="H1" s="129" t="s">
+      <c r="A1" s="150"/>
+      <c r="B1" s="151"/>
+      <c r="C1" s="151"/>
+      <c r="D1" s="151"/>
+      <c r="E1" s="151"/>
+      <c r="F1" s="151"/>
+      <c r="G1" s="152"/>
+      <c r="H1" s="199" t="s">
         <v>0</v>
       </c>
-      <c r="I1" s="130"/>
-      <c r="J1" s="130"/>
-      <c r="K1" s="130"/>
-      <c r="L1" s="130"/>
-      <c r="M1" s="130"/>
-      <c r="N1" s="130"/>
-      <c r="O1" s="130"/>
-      <c r="P1" s="130"/>
-      <c r="Q1" s="130"/>
-      <c r="R1" s="130"/>
-      <c r="S1" s="130"/>
-      <c r="T1" s="130"/>
-      <c r="U1" s="130"/>
-      <c r="V1" s="130"/>
-      <c r="W1" s="130"/>
-      <c r="X1" s="130"/>
-      <c r="Y1" s="130"/>
-      <c r="Z1" s="130"/>
-      <c r="AA1" s="131"/>
-      <c r="AB1" s="199"/>
-      <c r="AC1" s="200"/>
-      <c r="AD1" s="200"/>
-      <c r="AE1" s="201"/>
+      <c r="I1" s="200"/>
+      <c r="J1" s="200"/>
+      <c r="K1" s="200"/>
+      <c r="L1" s="200"/>
+      <c r="M1" s="200"/>
+      <c r="N1" s="200"/>
+      <c r="O1" s="200"/>
+      <c r="P1" s="200"/>
+      <c r="Q1" s="200"/>
+      <c r="R1" s="200"/>
+      <c r="S1" s="200"/>
+      <c r="T1" s="200"/>
+      <c r="U1" s="200"/>
+      <c r="V1" s="200"/>
+      <c r="W1" s="200"/>
+      <c r="X1" s="200"/>
+      <c r="Y1" s="200"/>
+      <c r="Z1" s="200"/>
+      <c r="AA1" s="201"/>
+      <c r="AB1" s="129"/>
+      <c r="AC1" s="130"/>
+      <c r="AD1" s="130"/>
+      <c r="AE1" s="131"/>
     </row>
     <row r="2" spans="1:31" ht="29.65" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="178"/>
-      <c r="B2" s="179"/>
-      <c r="C2" s="179"/>
-      <c r="D2" s="179"/>
-      <c r="E2" s="179"/>
-      <c r="F2" s="179"/>
-      <c r="G2" s="180"/>
+      <c r="A2" s="153"/>
+      <c r="B2" s="154"/>
+      <c r="C2" s="154"/>
+      <c r="D2" s="154"/>
+      <c r="E2" s="154"/>
+      <c r="F2" s="154"/>
+      <c r="G2" s="155"/>
       <c r="H2" s="68" t="s">
-        <v>32</v>
-      </c>
-      <c r="I2" s="132"/>
-      <c r="J2" s="132"/>
-      <c r="K2" s="132"/>
-      <c r="L2" s="132"/>
-      <c r="M2" s="132"/>
-      <c r="N2" s="132"/>
-      <c r="O2" s="133"/>
-      <c r="P2" s="187" t="s">
+        <v>31</v>
+      </c>
+      <c r="I2" s="202"/>
+      <c r="J2" s="202"/>
+      <c r="K2" s="202"/>
+      <c r="L2" s="202"/>
+      <c r="M2" s="202"/>
+      <c r="N2" s="202"/>
+      <c r="O2" s="203"/>
+      <c r="P2" s="139" t="s">
         <v>4</v>
       </c>
-      <c r="Q2" s="188"/>
-      <c r="R2" s="185">
+      <c r="Q2" s="140"/>
+      <c r="R2" s="161">
         <v>43831</v>
       </c>
-      <c r="S2" s="185"/>
-      <c r="T2" s="185"/>
-      <c r="U2" s="185"/>
-      <c r="V2" s="186"/>
+      <c r="S2" s="161"/>
+      <c r="T2" s="161"/>
+      <c r="U2" s="161"/>
+      <c r="V2" s="162"/>
       <c r="W2" s="123" t="s">
         <v>5</v>
       </c>
-      <c r="X2" s="193" t="s">
-        <v>209</v>
-      </c>
-      <c r="Y2" s="193"/>
-      <c r="Z2" s="193"/>
-      <c r="AA2" s="194"/>
-      <c r="AB2" s="202"/>
-      <c r="AC2" s="203"/>
-      <c r="AD2" s="203"/>
-      <c r="AE2" s="204"/>
+      <c r="X2" s="173" t="s">
+        <v>208</v>
+      </c>
+      <c r="Y2" s="173"/>
+      <c r="Z2" s="173"/>
+      <c r="AA2" s="174"/>
+      <c r="AB2" s="132"/>
+      <c r="AC2" s="133"/>
+      <c r="AD2" s="133"/>
+      <c r="AE2" s="134"/>
     </row>
     <row r="3" spans="1:31" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="181"/>
-      <c r="B3" s="182"/>
-      <c r="C3" s="182"/>
-      <c r="D3" s="182"/>
-      <c r="E3" s="182"/>
-      <c r="F3" s="182"/>
-      <c r="G3" s="183"/>
+      <c r="A3" s="156"/>
+      <c r="B3" s="157"/>
+      <c r="C3" s="157"/>
+      <c r="D3" s="157"/>
+      <c r="E3" s="157"/>
+      <c r="F3" s="157"/>
+      <c r="G3" s="158"/>
       <c r="H3" s="68" t="s">
         <v>7</v>
       </c>
-      <c r="I3" s="132"/>
-      <c r="J3" s="132"/>
-      <c r="K3" s="132"/>
-      <c r="L3" s="132"/>
-      <c r="M3" s="132"/>
-      <c r="N3" s="132"/>
-      <c r="O3" s="133"/>
-      <c r="P3" s="134" t="s">
+      <c r="I3" s="202"/>
+      <c r="J3" s="202"/>
+      <c r="K3" s="202"/>
+      <c r="L3" s="202"/>
+      <c r="M3" s="202"/>
+      <c r="N3" s="202"/>
+      <c r="O3" s="203"/>
+      <c r="P3" s="204" t="s">
         <v>26</v>
       </c>
-      <c r="Q3" s="135"/>
-      <c r="R3" s="173">
+      <c r="Q3" s="205"/>
+      <c r="R3" s="210">
         <v>1</v>
       </c>
-      <c r="S3" s="173"/>
-      <c r="T3" s="173"/>
-      <c r="U3" s="173"/>
-      <c r="V3" s="174"/>
-      <c r="W3" s="157" t="s">
+      <c r="S3" s="210"/>
+      <c r="T3" s="210"/>
+      <c r="U3" s="210"/>
+      <c r="V3" s="211"/>
+      <c r="W3" s="208" t="s">
         <v>6</v>
       </c>
-      <c r="X3" s="158"/>
-      <c r="Y3" s="155">
+      <c r="X3" s="209"/>
+      <c r="Y3" s="206">
         <v>43800</v>
       </c>
-      <c r="Z3" s="155"/>
-      <c r="AA3" s="156"/>
-      <c r="AB3" s="205"/>
-      <c r="AC3" s="206"/>
-      <c r="AD3" s="206"/>
-      <c r="AE3" s="207"/>
+      <c r="Z3" s="206"/>
+      <c r="AA3" s="207"/>
+      <c r="AB3" s="135"/>
+      <c r="AC3" s="136"/>
+      <c r="AD3" s="136"/>
+      <c r="AE3" s="137"/>
     </row>
     <row r="4" spans="1:31" ht="13.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="69"/>
@@ -3950,39 +3953,39 @@
       <c r="AE4" s="124"/>
     </row>
     <row r="5" spans="1:31" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="149" t="s">
+      <c r="A5" s="168" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="150"/>
-      <c r="C5" s="150"/>
-      <c r="D5" s="150"/>
-      <c r="E5" s="150"/>
-      <c r="F5" s="150"/>
-      <c r="G5" s="150"/>
-      <c r="H5" s="150"/>
-      <c r="I5" s="150"/>
-      <c r="J5" s="150"/>
-      <c r="K5" s="150"/>
-      <c r="L5" s="150"/>
-      <c r="M5" s="150"/>
-      <c r="N5" s="150"/>
-      <c r="O5" s="150"/>
-      <c r="P5" s="150"/>
-      <c r="Q5" s="150"/>
-      <c r="R5" s="150"/>
-      <c r="S5" s="150"/>
-      <c r="T5" s="150"/>
-      <c r="U5" s="150"/>
-      <c r="V5" s="150"/>
-      <c r="W5" s="150"/>
-      <c r="X5" s="150"/>
-      <c r="Y5" s="150"/>
-      <c r="Z5" s="150"/>
-      <c r="AA5" s="150"/>
-      <c r="AB5" s="150"/>
-      <c r="AC5" s="150"/>
-      <c r="AD5" s="150"/>
-      <c r="AE5" s="192"/>
+      <c r="B5" s="169"/>
+      <c r="C5" s="169"/>
+      <c r="D5" s="169"/>
+      <c r="E5" s="169"/>
+      <c r="F5" s="169"/>
+      <c r="G5" s="169"/>
+      <c r="H5" s="169"/>
+      <c r="I5" s="169"/>
+      <c r="J5" s="169"/>
+      <c r="K5" s="169"/>
+      <c r="L5" s="169"/>
+      <c r="M5" s="169"/>
+      <c r="N5" s="169"/>
+      <c r="O5" s="169"/>
+      <c r="P5" s="169"/>
+      <c r="Q5" s="169"/>
+      <c r="R5" s="169"/>
+      <c r="S5" s="169"/>
+      <c r="T5" s="169"/>
+      <c r="U5" s="169"/>
+      <c r="V5" s="169"/>
+      <c r="W5" s="169"/>
+      <c r="X5" s="169"/>
+      <c r="Y5" s="169"/>
+      <c r="Z5" s="169"/>
+      <c r="AA5" s="169"/>
+      <c r="AB5" s="169"/>
+      <c r="AC5" s="169"/>
+      <c r="AD5" s="169"/>
+      <c r="AE5" s="170"/>
     </row>
     <row r="6" spans="1:31" ht="7.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="74"/>
@@ -4019,49 +4022,49 @@
     </row>
     <row r="7" spans="1:31" ht="25.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="74"/>
-      <c r="B7" s="159" t="s">
+      <c r="B7" s="179" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="159"/>
-      <c r="D7" s="159"/>
-      <c r="E7" s="159"/>
-      <c r="F7" s="159"/>
-      <c r="G7" s="160"/>
-      <c r="H7" s="136" t="s">
+      <c r="C7" s="179"/>
+      <c r="D7" s="179"/>
+      <c r="E7" s="179"/>
+      <c r="F7" s="179"/>
+      <c r="G7" s="180"/>
+      <c r="H7" s="187" t="s">
         <v>17</v>
       </c>
-      <c r="I7" s="137"/>
-      <c r="J7" s="138"/>
+      <c r="I7" s="188"/>
+      <c r="J7" s="189"/>
       <c r="K7" s="119" t="s">
         <v>18</v>
       </c>
-      <c r="L7" s="136">
+      <c r="L7" s="187">
         <v>20508972734</v>
       </c>
-      <c r="M7" s="137"/>
-      <c r="N7" s="138"/>
-      <c r="O7" s="198" t="s">
+      <c r="M7" s="188"/>
+      <c r="N7" s="189"/>
+      <c r="O7" s="178" t="s">
         <v>19</v>
       </c>
-      <c r="P7" s="159"/>
-      <c r="Q7" s="160"/>
-      <c r="R7" s="195" t="s">
+      <c r="P7" s="179"/>
+      <c r="Q7" s="180"/>
+      <c r="R7" s="175" t="s">
         <v>20</v>
       </c>
-      <c r="S7" s="196"/>
-      <c r="T7" s="196"/>
-      <c r="U7" s="196"/>
-      <c r="V7" s="197"/>
+      <c r="S7" s="176"/>
+      <c r="T7" s="176"/>
+      <c r="U7" s="176"/>
+      <c r="V7" s="177"/>
       <c r="W7" s="77"/>
       <c r="X7" s="120" t="s">
         <v>21</v>
       </c>
-      <c r="Y7" s="195"/>
-      <c r="Z7" s="196"/>
-      <c r="AA7" s="196"/>
-      <c r="AB7" s="196"/>
-      <c r="AC7" s="196"/>
-      <c r="AD7" s="197"/>
+      <c r="Y7" s="175"/>
+      <c r="Z7" s="176"/>
+      <c r="AA7" s="176"/>
+      <c r="AB7" s="176"/>
+      <c r="AC7" s="176"/>
+      <c r="AD7" s="177"/>
       <c r="AE7" s="78"/>
     </row>
     <row r="8" spans="1:31" ht="7.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -4130,39 +4133,39 @@
       <c r="AE9" s="86"/>
     </row>
     <row r="10" spans="1:31" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="149" t="s">
+      <c r="A10" s="168" t="s">
         <v>22</v>
       </c>
-      <c r="B10" s="150"/>
-      <c r="C10" s="150"/>
-      <c r="D10" s="150"/>
-      <c r="E10" s="150"/>
-      <c r="F10" s="150"/>
-      <c r="G10" s="150"/>
-      <c r="H10" s="150"/>
-      <c r="I10" s="150"/>
-      <c r="J10" s="150"/>
-      <c r="K10" s="150"/>
-      <c r="L10" s="150"/>
-      <c r="M10" s="150"/>
-      <c r="N10" s="150"/>
-      <c r="O10" s="150"/>
-      <c r="P10" s="150"/>
-      <c r="Q10" s="150"/>
-      <c r="R10" s="150"/>
-      <c r="S10" s="150"/>
-      <c r="T10" s="150"/>
-      <c r="U10" s="150"/>
-      <c r="V10" s="150"/>
-      <c r="W10" s="150"/>
-      <c r="X10" s="150"/>
-      <c r="Y10" s="150"/>
-      <c r="Z10" s="150"/>
-      <c r="AA10" s="150"/>
-      <c r="AB10" s="150"/>
-      <c r="AC10" s="150"/>
-      <c r="AD10" s="150"/>
-      <c r="AE10" s="192"/>
+      <c r="B10" s="169"/>
+      <c r="C10" s="169"/>
+      <c r="D10" s="169"/>
+      <c r="E10" s="169"/>
+      <c r="F10" s="169"/>
+      <c r="G10" s="169"/>
+      <c r="H10" s="169"/>
+      <c r="I10" s="169"/>
+      <c r="J10" s="169"/>
+      <c r="K10" s="169"/>
+      <c r="L10" s="169"/>
+      <c r="M10" s="169"/>
+      <c r="N10" s="169"/>
+      <c r="O10" s="169"/>
+      <c r="P10" s="169"/>
+      <c r="Q10" s="169"/>
+      <c r="R10" s="169"/>
+      <c r="S10" s="169"/>
+      <c r="T10" s="169"/>
+      <c r="U10" s="169"/>
+      <c r="V10" s="169"/>
+      <c r="W10" s="169"/>
+      <c r="X10" s="169"/>
+      <c r="Y10" s="169"/>
+      <c r="Z10" s="169"/>
+      <c r="AA10" s="169"/>
+      <c r="AB10" s="169"/>
+      <c r="AC10" s="169"/>
+      <c r="AD10" s="169"/>
+      <c r="AE10" s="170"/>
     </row>
     <row r="11" spans="1:31" ht="7.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="87"/>
@@ -4196,41 +4199,41 @@
     </row>
     <row r="12" spans="1:31" ht="37.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="74"/>
-      <c r="B12" s="151" t="s">
+      <c r="B12" s="163" t="s">
+        <v>287</v>
+      </c>
+      <c r="C12" s="163"/>
+      <c r="D12" s="163"/>
+      <c r="E12" s="163"/>
+      <c r="F12" s="163"/>
+      <c r="G12" s="164"/>
+      <c r="H12" s="181"/>
+      <c r="I12" s="185"/>
+      <c r="J12" s="185"/>
+      <c r="K12" s="185"/>
+      <c r="L12" s="182"/>
+      <c r="M12" s="190" t="s">
         <v>288</v>
       </c>
-      <c r="C12" s="151"/>
-      <c r="D12" s="151"/>
-      <c r="E12" s="151"/>
-      <c r="F12" s="151"/>
-      <c r="G12" s="152"/>
-      <c r="H12" s="164"/>
-      <c r="I12" s="169"/>
-      <c r="J12" s="169"/>
-      <c r="K12" s="169"/>
-      <c r="L12" s="165"/>
-      <c r="M12" s="171" t="s">
-        <v>289</v>
-      </c>
-      <c r="N12" s="168"/>
-      <c r="O12" s="172"/>
-      <c r="P12" s="161"/>
-      <c r="Q12" s="162"/>
-      <c r="R12" s="162"/>
-      <c r="S12" s="162"/>
-      <c r="T12" s="163"/>
-      <c r="U12" s="189" t="s">
-        <v>211</v>
-      </c>
-      <c r="V12" s="190"/>
-      <c r="W12" s="190"/>
-      <c r="X12" s="191"/>
-      <c r="Y12" s="166"/>
-      <c r="Z12" s="170"/>
-      <c r="AA12" s="170"/>
-      <c r="AB12" s="170"/>
-      <c r="AC12" s="170"/>
-      <c r="AD12" s="167"/>
+      <c r="N12" s="147"/>
+      <c r="O12" s="148"/>
+      <c r="P12" s="171"/>
+      <c r="Q12" s="149"/>
+      <c r="R12" s="149"/>
+      <c r="S12" s="149"/>
+      <c r="T12" s="172"/>
+      <c r="U12" s="165" t="s">
+        <v>210</v>
+      </c>
+      <c r="V12" s="166"/>
+      <c r="W12" s="166"/>
+      <c r="X12" s="167"/>
+      <c r="Y12" s="183"/>
+      <c r="Z12" s="186"/>
+      <c r="AA12" s="186"/>
+      <c r="AB12" s="186"/>
+      <c r="AC12" s="186"/>
+      <c r="AD12" s="184"/>
       <c r="AE12" s="90"/>
     </row>
     <row r="13" spans="1:31" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.2">
@@ -4268,43 +4271,43 @@
     </row>
     <row r="14" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A14" s="74"/>
-      <c r="B14" s="151" t="s">
+      <c r="B14" s="163" t="s">
         <v>23</v>
       </c>
-      <c r="C14" s="151"/>
-      <c r="D14" s="151"/>
-      <c r="E14" s="151"/>
-      <c r="F14" s="151"/>
-      <c r="G14" s="152"/>
-      <c r="H14" s="166"/>
-      <c r="I14" s="170"/>
-      <c r="J14" s="170"/>
-      <c r="K14" s="170"/>
-      <c r="L14" s="167"/>
+      <c r="C14" s="163"/>
+      <c r="D14" s="163"/>
+      <c r="E14" s="163"/>
+      <c r="F14" s="163"/>
+      <c r="G14" s="164"/>
+      <c r="H14" s="183"/>
+      <c r="I14" s="186"/>
+      <c r="J14" s="186"/>
+      <c r="K14" s="186"/>
+      <c r="L14" s="184"/>
       <c r="M14" s="86"/>
       <c r="N14" s="86"/>
       <c r="O14" s="85" t="s">
         <v>24</v>
       </c>
-      <c r="P14" s="164"/>
-      <c r="Q14" s="165"/>
+      <c r="P14" s="181"/>
+      <c r="Q14" s="182"/>
       <c r="R14" s="122" t="s">
         <v>25</v>
       </c>
-      <c r="S14" s="166"/>
-      <c r="T14" s="167"/>
+      <c r="S14" s="183"/>
+      <c r="T14" s="184"/>
       <c r="U14" s="121"/>
-      <c r="V14" s="168" t="s">
+      <c r="V14" s="147" t="s">
         <v>14</v>
       </c>
-      <c r="W14" s="168"/>
-      <c r="X14" s="168"/>
-      <c r="Y14" s="208"/>
-      <c r="Z14" s="208"/>
-      <c r="AA14" s="208"/>
-      <c r="AB14" s="208"/>
-      <c r="AC14" s="208"/>
-      <c r="AD14" s="208"/>
+      <c r="W14" s="147"/>
+      <c r="X14" s="147"/>
+      <c r="Y14" s="224"/>
+      <c r="Z14" s="224"/>
+      <c r="AA14" s="224"/>
+      <c r="AB14" s="138"/>
+      <c r="AC14" s="138"/>
+      <c r="AD14" s="138"/>
       <c r="AE14" s="95"/>
     </row>
     <row r="15" spans="1:31" x14ac:dyDescent="0.2">
@@ -4342,39 +4345,39 @@
     </row>
     <row r="16" spans="1:31" ht="46.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="74"/>
-      <c r="B16" s="151" t="s">
-        <v>287</v>
-      </c>
-      <c r="C16" s="151"/>
-      <c r="D16" s="151"/>
-      <c r="E16" s="151"/>
-      <c r="F16" s="151"/>
-      <c r="G16" s="152"/>
-      <c r="H16" s="184"/>
-      <c r="I16" s="184"/>
-      <c r="J16" s="184"/>
-      <c r="K16" s="184"/>
-      <c r="L16" s="184"/>
-      <c r="M16" s="184"/>
-      <c r="N16" s="184"/>
-      <c r="O16" s="184"/>
-      <c r="P16" s="184"/>
-      <c r="Q16" s="184"/>
-      <c r="R16" s="184"/>
+      <c r="B16" s="163" t="s">
+        <v>286</v>
+      </c>
+      <c r="C16" s="163"/>
+      <c r="D16" s="163"/>
+      <c r="E16" s="163"/>
+      <c r="F16" s="163"/>
+      <c r="G16" s="164"/>
+      <c r="H16" s="160"/>
+      <c r="I16" s="160"/>
+      <c r="J16" s="160"/>
+      <c r="K16" s="160"/>
+      <c r="L16" s="160"/>
+      <c r="M16" s="160"/>
+      <c r="N16" s="160"/>
+      <c r="O16" s="160"/>
+      <c r="P16" s="160"/>
+      <c r="Q16" s="160"/>
+      <c r="R16" s="160"/>
       <c r="S16" s="96"/>
-      <c r="T16" s="210" t="s">
-        <v>286</v>
-      </c>
-      <c r="U16" s="210"/>
-      <c r="V16" s="210"/>
-      <c r="W16" s="210"/>
-      <c r="X16" s="211"/>
-      <c r="Y16" s="187"/>
-      <c r="Z16" s="188"/>
-      <c r="AA16" s="188"/>
-      <c r="AB16" s="188"/>
-      <c r="AC16" s="188"/>
-      <c r="AD16" s="209"/>
+      <c r="T16" s="145" t="s">
+        <v>285</v>
+      </c>
+      <c r="U16" s="145"/>
+      <c r="V16" s="145"/>
+      <c r="W16" s="145"/>
+      <c r="X16" s="146"/>
+      <c r="Y16" s="139"/>
+      <c r="Z16" s="140"/>
+      <c r="AA16" s="140"/>
+      <c r="AB16" s="140"/>
+      <c r="AC16" s="140"/>
+      <c r="AD16" s="141"/>
       <c r="AE16" s="97"/>
     </row>
     <row r="17" spans="1:31" x14ac:dyDescent="0.2">
@@ -4412,38 +4415,38 @@
     </row>
     <row r="18" spans="1:31" ht="48.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="74"/>
-      <c r="B18" s="151" t="s">
+      <c r="B18" s="163" t="s">
         <v>13</v>
       </c>
-      <c r="C18" s="151"/>
-      <c r="D18" s="151"/>
-      <c r="E18" s="151"/>
-      <c r="F18" s="151"/>
-      <c r="G18" s="152"/>
-      <c r="H18" s="153"/>
-      <c r="I18" s="153"/>
-      <c r="J18" s="153"/>
-      <c r="K18" s="153"/>
-      <c r="L18" s="153"/>
-      <c r="M18" s="153"/>
-      <c r="N18" s="153"/>
-      <c r="O18" s="153"/>
-      <c r="P18" s="153"/>
-      <c r="Q18" s="153"/>
-      <c r="R18" s="153"/>
-      <c r="T18" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="U18" s="168"/>
-      <c r="V18" s="168"/>
-      <c r="W18" s="168"/>
-      <c r="X18" s="172"/>
-      <c r="Y18" s="161"/>
-      <c r="Z18" s="162"/>
-      <c r="AA18" s="162"/>
-      <c r="AB18" s="162"/>
-      <c r="AC18" s="162"/>
-      <c r="AD18" s="163"/>
+      <c r="C18" s="163"/>
+      <c r="D18" s="163"/>
+      <c r="E18" s="163"/>
+      <c r="F18" s="163"/>
+      <c r="G18" s="164"/>
+      <c r="H18" s="159"/>
+      <c r="I18" s="159"/>
+      <c r="J18" s="159"/>
+      <c r="K18" s="159"/>
+      <c r="L18" s="159"/>
+      <c r="M18" s="159"/>
+      <c r="N18" s="159"/>
+      <c r="O18" s="159"/>
+      <c r="P18" s="159"/>
+      <c r="Q18" s="159"/>
+      <c r="R18" s="159"/>
+      <c r="T18" s="147" t="s">
+        <v>292</v>
+      </c>
+      <c r="U18" s="147"/>
+      <c r="V18" s="147"/>
+      <c r="W18" s="147"/>
+      <c r="X18" s="148"/>
+      <c r="Y18" s="171"/>
+      <c r="Z18" s="149"/>
+      <c r="AA18" s="149"/>
+      <c r="AB18" s="149"/>
+      <c r="AC18" s="149"/>
+      <c r="AD18" s="172"/>
       <c r="AE18" s="98"/>
     </row>
     <row r="19" spans="1:31" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.2">
@@ -4481,37 +4484,37 @@
     </row>
     <row r="20" spans="1:31" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="74"/>
-      <c r="B20" s="151" t="s">
-        <v>28</v>
-      </c>
-      <c r="C20" s="151"/>
-      <c r="D20" s="151"/>
-      <c r="E20" s="151"/>
-      <c r="F20" s="151"/>
-      <c r="G20" s="152"/>
-      <c r="H20" s="141"/>
-      <c r="I20" s="142"/>
-      <c r="J20" s="142"/>
-      <c r="K20" s="142"/>
-      <c r="L20" s="142"/>
-      <c r="M20" s="142"/>
-      <c r="N20" s="142"/>
-      <c r="O20" s="142"/>
-      <c r="P20" s="142"/>
-      <c r="Q20" s="142"/>
-      <c r="R20" s="142"/>
-      <c r="S20" s="142"/>
-      <c r="T20" s="142"/>
-      <c r="U20" s="142"/>
-      <c r="V20" s="142"/>
-      <c r="W20" s="142"/>
-      <c r="X20" s="142"/>
-      <c r="Y20" s="142"/>
-      <c r="Z20" s="142"/>
-      <c r="AA20" s="142"/>
-      <c r="AB20" s="142"/>
-      <c r="AC20" s="142"/>
-      <c r="AD20" s="143"/>
+      <c r="B20" s="163" t="s">
+        <v>27</v>
+      </c>
+      <c r="C20" s="163"/>
+      <c r="D20" s="163"/>
+      <c r="E20" s="163"/>
+      <c r="F20" s="163"/>
+      <c r="G20" s="164"/>
+      <c r="H20" s="191"/>
+      <c r="I20" s="192"/>
+      <c r="J20" s="192"/>
+      <c r="K20" s="192"/>
+      <c r="L20" s="192"/>
+      <c r="M20" s="192"/>
+      <c r="N20" s="192"/>
+      <c r="O20" s="192"/>
+      <c r="P20" s="192"/>
+      <c r="Q20" s="192"/>
+      <c r="R20" s="192"/>
+      <c r="S20" s="192"/>
+      <c r="T20" s="192"/>
+      <c r="U20" s="192"/>
+      <c r="V20" s="192"/>
+      <c r="W20" s="192"/>
+      <c r="X20" s="192"/>
+      <c r="Y20" s="192"/>
+      <c r="Z20" s="192"/>
+      <c r="AA20" s="192"/>
+      <c r="AB20" s="192"/>
+      <c r="AC20" s="192"/>
+      <c r="AD20" s="193"/>
       <c r="AE20" s="99"/>
     </row>
     <row r="21" spans="1:31" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.2">
@@ -4549,41 +4552,41 @@
     </row>
     <row r="22" spans="1:31" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="74"/>
-      <c r="B22" s="151" t="s">
-        <v>283</v>
-      </c>
-      <c r="C22" s="151"/>
-      <c r="D22" s="151"/>
-      <c r="E22" s="151"/>
-      <c r="F22" s="151"/>
-      <c r="G22" s="152"/>
-      <c r="H22" s="153" t="s">
-        <v>290</v>
-      </c>
-      <c r="I22" s="153"/>
-      <c r="J22" s="153"/>
-      <c r="K22" s="153"/>
-      <c r="L22" s="153"/>
-      <c r="M22" s="153"/>
-      <c r="N22" s="153"/>
-      <c r="O22" s="153"/>
-      <c r="P22" s="153"/>
-      <c r="Q22" s="153"/>
-      <c r="R22" s="153"/>
+      <c r="B22" s="163" t="s">
+        <v>282</v>
+      </c>
+      <c r="C22" s="163"/>
+      <c r="D22" s="163"/>
+      <c r="E22" s="163"/>
+      <c r="F22" s="163"/>
+      <c r="G22" s="164"/>
+      <c r="H22" s="159" t="s">
+        <v>289</v>
+      </c>
+      <c r="I22" s="159"/>
+      <c r="J22" s="159"/>
+      <c r="K22" s="159"/>
+      <c r="L22" s="159"/>
+      <c r="M22" s="159"/>
+      <c r="N22" s="159"/>
+      <c r="O22" s="159"/>
+      <c r="P22" s="159"/>
+      <c r="Q22" s="159"/>
+      <c r="R22" s="159"/>
       <c r="S22" s="127"/>
       <c r="T22" s="127"/>
       <c r="U22" s="127"/>
       <c r="V22" s="127"/>
       <c r="W22" s="85" t="s">
-        <v>291</v>
-      </c>
-      <c r="X22" s="154"/>
-      <c r="Y22" s="154"/>
-      <c r="Z22" s="154"/>
-      <c r="AA22" s="154"/>
-      <c r="AB22" s="154"/>
-      <c r="AC22" s="154"/>
-      <c r="AD22" s="154"/>
+        <v>290</v>
+      </c>
+      <c r="X22" s="198"/>
+      <c r="Y22" s="198"/>
+      <c r="Z22" s="198"/>
+      <c r="AA22" s="198"/>
+      <c r="AB22" s="198"/>
+      <c r="AC22" s="198"/>
+      <c r="AD22" s="198"/>
       <c r="AE22" s="99"/>
     </row>
     <row r="23" spans="1:31" ht="7.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -4622,43 +4625,43 @@
     <row r="24" spans="1:31" ht="13.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D24" s="117"/>
       <c r="E24" s="117"/>
-      <c r="F24" s="162"/>
-      <c r="G24" s="162"/>
-      <c r="H24" s="162"/>
-      <c r="I24" s="162"/>
-      <c r="J24" s="162"/>
-      <c r="K24" s="162"/>
-      <c r="L24" s="162"/>
-      <c r="M24" s="162"/>
-      <c r="N24" s="162"/>
-      <c r="O24" s="162"/>
-      <c r="P24" s="162"/>
-      <c r="Q24" s="162"/>
-      <c r="R24" s="162"/>
-      <c r="S24" s="162"/>
-      <c r="T24" s="162"/>
-      <c r="U24" s="162"/>
-      <c r="V24" s="162"/>
-      <c r="W24" s="162"/>
-      <c r="X24" s="162"/>
-      <c r="Y24" s="162"/>
-      <c r="Z24" s="162"/>
-      <c r="AA24" s="162"/>
-      <c r="AB24" s="162"/>
-      <c r="AC24" s="162"/>
-      <c r="AD24" s="162"/>
-      <c r="AE24" s="162"/>
+      <c r="F24" s="149"/>
+      <c r="G24" s="149"/>
+      <c r="H24" s="149"/>
+      <c r="I24" s="149"/>
+      <c r="J24" s="149"/>
+      <c r="K24" s="149"/>
+      <c r="L24" s="149"/>
+      <c r="M24" s="149"/>
+      <c r="N24" s="149"/>
+      <c r="O24" s="149"/>
+      <c r="P24" s="149"/>
+      <c r="Q24" s="149"/>
+      <c r="R24" s="149"/>
+      <c r="S24" s="149"/>
+      <c r="T24" s="149"/>
+      <c r="U24" s="149"/>
+      <c r="V24" s="149"/>
+      <c r="W24" s="149"/>
+      <c r="X24" s="149"/>
+      <c r="Y24" s="149"/>
+      <c r="Z24" s="149"/>
+      <c r="AA24" s="149"/>
+      <c r="AB24" s="149"/>
+      <c r="AC24" s="149"/>
+      <c r="AD24" s="149"/>
+      <c r="AE24" s="149"/>
     </row>
     <row r="25" spans="1:31" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="149" t="s">
-        <v>30</v>
-      </c>
-      <c r="B25" s="150"/>
-      <c r="C25" s="150"/>
-      <c r="D25" s="150"/>
-      <c r="E25" s="150"/>
-      <c r="F25" s="150"/>
-      <c r="G25" s="150"/>
+      <c r="A25" s="168" t="s">
+        <v>29</v>
+      </c>
+      <c r="B25" s="169"/>
+      <c r="C25" s="169"/>
+      <c r="D25" s="169"/>
+      <c r="E25" s="169"/>
+      <c r="F25" s="169"/>
+      <c r="G25" s="169"/>
       <c r="H25" s="103"/>
       <c r="I25" s="103"/>
       <c r="J25" s="103"/>
@@ -4685,96 +4688,96 @@
       <c r="AE25" s="104"/>
     </row>
     <row r="26" spans="1:31" ht="3.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="145"/>
-      <c r="B26" s="146"/>
-      <c r="C26" s="146"/>
-      <c r="D26" s="146"/>
-      <c r="E26" s="146"/>
-      <c r="F26" s="146"/>
-      <c r="G26" s="146"/>
-      <c r="H26" s="146"/>
-      <c r="I26" s="146"/>
-      <c r="J26" s="146"/>
-      <c r="K26" s="146"/>
-      <c r="L26" s="146"/>
-      <c r="M26" s="146"/>
-      <c r="N26" s="146"/>
-      <c r="O26" s="146"/>
-      <c r="P26" s="146"/>
-      <c r="Q26" s="146"/>
-      <c r="R26" s="146"/>
-      <c r="S26" s="146"/>
-      <c r="T26" s="146"/>
-      <c r="U26" s="146"/>
-      <c r="V26" s="146"/>
-      <c r="W26" s="146"/>
-      <c r="X26" s="146"/>
-      <c r="Y26" s="146"/>
-      <c r="Z26" s="146"/>
-      <c r="AA26" s="146"/>
-      <c r="AB26" s="146"/>
-      <c r="AC26" s="146"/>
-      <c r="AD26" s="146"/>
-      <c r="AE26" s="147"/>
+      <c r="A26" s="195"/>
+      <c r="B26" s="196"/>
+      <c r="C26" s="196"/>
+      <c r="D26" s="196"/>
+      <c r="E26" s="196"/>
+      <c r="F26" s="196"/>
+      <c r="G26" s="196"/>
+      <c r="H26" s="196"/>
+      <c r="I26" s="196"/>
+      <c r="J26" s="196"/>
+      <c r="K26" s="196"/>
+      <c r="L26" s="196"/>
+      <c r="M26" s="196"/>
+      <c r="N26" s="196"/>
+      <c r="O26" s="196"/>
+      <c r="P26" s="196"/>
+      <c r="Q26" s="196"/>
+      <c r="R26" s="196"/>
+      <c r="S26" s="196"/>
+      <c r="T26" s="196"/>
+      <c r="U26" s="196"/>
+      <c r="V26" s="196"/>
+      <c r="W26" s="196"/>
+      <c r="X26" s="196"/>
+      <c r="Y26" s="196"/>
+      <c r="Z26" s="196"/>
+      <c r="AA26" s="196"/>
+      <c r="AB26" s="196"/>
+      <c r="AC26" s="196"/>
+      <c r="AD26" s="196"/>
+      <c r="AE26" s="197"/>
     </row>
     <row r="27" spans="1:31" ht="52.9" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="139" t="s">
+      <c r="A27" s="142" t="s">
         <v>1</v>
       </c>
-      <c r="B27" s="140"/>
+      <c r="B27" s="144"/>
       <c r="C27" s="105" t="s">
         <v>8</v>
       </c>
-      <c r="D27" s="139" t="s">
+      <c r="D27" s="142" t="s">
         <v>9</v>
       </c>
-      <c r="E27" s="148"/>
-      <c r="F27" s="148"/>
-      <c r="G27" s="148"/>
-      <c r="H27" s="148"/>
-      <c r="I27" s="140"/>
-      <c r="J27" s="139" t="s">
+      <c r="E27" s="143"/>
+      <c r="F27" s="143"/>
+      <c r="G27" s="143"/>
+      <c r="H27" s="143"/>
+      <c r="I27" s="144"/>
+      <c r="J27" s="142" t="s">
         <v>10</v>
       </c>
-      <c r="K27" s="148"/>
-      <c r="L27" s="139" t="s">
-        <v>29</v>
-      </c>
-      <c r="M27" s="148"/>
-      <c r="N27" s="140"/>
-      <c r="O27" s="139" t="s">
-        <v>285</v>
-      </c>
-      <c r="P27" s="148"/>
-      <c r="Q27" s="140"/>
+      <c r="K27" s="143"/>
+      <c r="L27" s="142" t="s">
+        <v>28</v>
+      </c>
+      <c r="M27" s="143"/>
+      <c r="N27" s="144"/>
+      <c r="O27" s="142" t="s">
+        <v>284</v>
+      </c>
+      <c r="P27" s="143"/>
+      <c r="Q27" s="144"/>
       <c r="R27" s="105" t="s">
         <v>2</v>
       </c>
-      <c r="S27" s="139" t="s">
-        <v>284</v>
-      </c>
-      <c r="T27" s="148"/>
-      <c r="U27" s="148"/>
-      <c r="V27" s="148"/>
+      <c r="S27" s="142" t="s">
+        <v>283</v>
+      </c>
+      <c r="T27" s="143"/>
+      <c r="U27" s="143"/>
+      <c r="V27" s="143"/>
       <c r="W27" s="105" t="s">
         <v>11</v>
       </c>
       <c r="X27" s="105" t="s">
         <v>3</v>
       </c>
-      <c r="Y27" s="139" t="s">
+      <c r="Y27" s="142" t="s">
         <v>12</v>
       </c>
-      <c r="Z27" s="148"/>
-      <c r="AA27" s="148"/>
-      <c r="AB27" s="140"/>
+      <c r="Z27" s="143"/>
+      <c r="AA27" s="143"/>
+      <c r="AB27" s="144"/>
       <c r="AC27" s="128" t="s">
-        <v>31</v>
-      </c>
-      <c r="AD27" s="144" t="s">
-        <v>292</v>
-      </c>
-      <c r="AE27" s="144"/>
+        <v>30</v>
+      </c>
+      <c r="AD27" s="194" t="s">
+        <v>291</v>
+      </c>
+      <c r="AE27" s="194"/>
     </row>
     <row r="28" spans="1:31" ht="13.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="116"/>
@@ -6945,6 +6948,47 @@
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" selectLockedCells="1" sort="0" autoFilter="0" pivotTables="0"/>
   <mergeCells count="57">
+    <mergeCell ref="H1:AA1"/>
+    <mergeCell ref="I2:O2"/>
+    <mergeCell ref="I3:O3"/>
+    <mergeCell ref="P3:Q3"/>
+    <mergeCell ref="L7:N7"/>
+    <mergeCell ref="Y3:AA3"/>
+    <mergeCell ref="W3:X3"/>
+    <mergeCell ref="R3:V3"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="H20:AD20"/>
+    <mergeCell ref="AD27:AE27"/>
+    <mergeCell ref="A26:AE26"/>
+    <mergeCell ref="D27:I27"/>
+    <mergeCell ref="A25:G25"/>
+    <mergeCell ref="B22:G22"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="L27:N27"/>
+    <mergeCell ref="H22:R22"/>
+    <mergeCell ref="X22:AD22"/>
+    <mergeCell ref="O27:Q27"/>
+    <mergeCell ref="Y18:AD18"/>
+    <mergeCell ref="P14:Q14"/>
+    <mergeCell ref="S14:T14"/>
+    <mergeCell ref="V14:X14"/>
+    <mergeCell ref="B12:G12"/>
+    <mergeCell ref="H12:L12"/>
+    <mergeCell ref="H14:L14"/>
+    <mergeCell ref="B14:G14"/>
+    <mergeCell ref="Y12:AD12"/>
+    <mergeCell ref="M12:O12"/>
+    <mergeCell ref="X2:AA2"/>
+    <mergeCell ref="Y7:AD7"/>
+    <mergeCell ref="R7:V7"/>
+    <mergeCell ref="O7:Q7"/>
+    <mergeCell ref="B7:G7"/>
+    <mergeCell ref="H7:J7"/>
+    <mergeCell ref="U12:X12"/>
+    <mergeCell ref="A5:AE5"/>
+    <mergeCell ref="A10:AE10"/>
+    <mergeCell ref="B16:G16"/>
+    <mergeCell ref="P12:T12"/>
     <mergeCell ref="AB1:AE3"/>
     <mergeCell ref="AB14:AD14"/>
     <mergeCell ref="Y16:AD16"/>
@@ -6961,47 +7005,6 @@
     <mergeCell ref="B20:G20"/>
     <mergeCell ref="B18:G18"/>
     <mergeCell ref="P2:Q2"/>
-    <mergeCell ref="U12:X12"/>
-    <mergeCell ref="A5:AE5"/>
-    <mergeCell ref="A10:AE10"/>
-    <mergeCell ref="B16:G16"/>
-    <mergeCell ref="P12:T12"/>
-    <mergeCell ref="X2:AA2"/>
-    <mergeCell ref="Y7:AD7"/>
-    <mergeCell ref="R7:V7"/>
-    <mergeCell ref="O7:Q7"/>
-    <mergeCell ref="B7:G7"/>
-    <mergeCell ref="Y18:AD18"/>
-    <mergeCell ref="P14:Q14"/>
-    <mergeCell ref="S14:T14"/>
-    <mergeCell ref="V14:X14"/>
-    <mergeCell ref="B12:G12"/>
-    <mergeCell ref="H12:L12"/>
-    <mergeCell ref="H14:L14"/>
-    <mergeCell ref="H7:J7"/>
-    <mergeCell ref="B14:G14"/>
-    <mergeCell ref="Y12:AD12"/>
-    <mergeCell ref="M12:O12"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="H20:AD20"/>
-    <mergeCell ref="AD27:AE27"/>
-    <mergeCell ref="A26:AE26"/>
-    <mergeCell ref="D27:I27"/>
-    <mergeCell ref="A25:G25"/>
-    <mergeCell ref="B22:G22"/>
-    <mergeCell ref="J27:K27"/>
-    <mergeCell ref="L27:N27"/>
-    <mergeCell ref="H22:R22"/>
-    <mergeCell ref="X22:AD22"/>
-    <mergeCell ref="O27:Q27"/>
-    <mergeCell ref="H1:AA1"/>
-    <mergeCell ref="I2:O2"/>
-    <mergeCell ref="I3:O3"/>
-    <mergeCell ref="P3:Q3"/>
-    <mergeCell ref="L7:N7"/>
-    <mergeCell ref="Y3:AA3"/>
-    <mergeCell ref="W3:X3"/>
-    <mergeCell ref="R3:V3"/>
   </mergeCells>
   <printOptions horizontalCentered="1" gridLinesSet="0"/>
   <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.19685039370078741" bottom="0.35433070866141736" header="0.11811023622047245" footer="0.19685039370078741"/>
@@ -7052,287 +7055,287 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="212" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B1" s="213"/>
       <c r="D1" s="212" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E1" s="213"/>
     </row>
     <row r="2" spans="1:5" s="4" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="B2" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="B2" s="5" t="s">
-        <v>114</v>
-      </c>
       <c r="D2" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="E2" s="5" t="s">
         <v>117</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="22.5" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="22.5" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="22.5" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="22.5" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="22.5" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="22.5" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="22.5" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="22.5" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="22.5" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B19" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="22.5" x14ac:dyDescent="0.25">
       <c r="B20" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B21" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B22" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B23" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -7877,7 +7880,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="217" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B1" s="218"/>
       <c r="C1" s="218"/>
@@ -7885,7 +7888,7 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="214" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B2" s="215"/>
       <c r="C2" s="215"/>
@@ -7893,59 +7896,59 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="34" t="s">
+        <v>194</v>
+      </c>
+      <c r="B3" s="34" t="s">
         <v>195</v>
       </c>
-      <c r="B3" s="34" t="s">
+      <c r="C3" s="34" t="s">
         <v>196</v>
       </c>
-      <c r="C3" s="34" t="s">
+      <c r="D3" s="34" t="s">
         <v>197</v>
-      </c>
-      <c r="D3" s="34" t="s">
-        <v>198</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="76.5" x14ac:dyDescent="0.2">
       <c r="A4" s="35" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B4" s="28">
         <v>3</v>
       </c>
       <c r="C4" s="26" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D4" s="27" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="76.5" x14ac:dyDescent="0.2">
       <c r="A5" s="35" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B5" s="28">
         <v>2</v>
       </c>
       <c r="C5" s="26" t="s">
+        <v>199</v>
+      </c>
+      <c r="D5" s="27" t="s">
         <v>200</v>
-      </c>
-      <c r="D5" s="27" t="s">
-        <v>201</v>
       </c>
       <c r="G5" s="36"/>
     </row>
     <row r="6" spans="1:8" ht="76.5" x14ac:dyDescent="0.2">
       <c r="A6" s="35" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B6" s="37">
         <v>1</v>
       </c>
       <c r="C6" s="26" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D6" s="27" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="G6" s="36"/>
     </row>
@@ -7957,7 +7960,7 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" s="214" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B8" s="215"/>
       <c r="C8" s="215"/>
@@ -7965,58 +7968,58 @@
     </row>
     <row r="9" spans="1:8" ht="23.65" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="34" t="s">
+        <v>194</v>
+      </c>
+      <c r="B9" s="34" t="s">
         <v>195</v>
       </c>
-      <c r="B9" s="34" t="s">
-        <v>196</v>
-      </c>
       <c r="C9" s="34" t="s">
+        <v>203</v>
+      </c>
+      <c r="D9" s="34" t="s">
         <v>204</v>
-      </c>
-      <c r="D9" s="34" t="s">
-        <v>205</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A10" s="35" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B10" s="28">
         <v>3</v>
       </c>
       <c r="C10" s="28" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D10" s="27" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A11" s="35" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B11" s="28">
         <v>2</v>
       </c>
       <c r="C11" s="28" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D11" s="27" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A12" s="35" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B12" s="28">
         <v>1</v>
       </c>
       <c r="C12" s="28" t="s">
+        <v>177</v>
+      </c>
+      <c r="D12" s="27" t="s">
         <v>178</v>
-      </c>
-      <c r="D12" s="27" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
@@ -8027,7 +8030,7 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" s="214" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B14" s="215"/>
       <c r="C14" s="215"/>
@@ -8065,16 +8068,16 @@
       <c r="E19" s="38"/>
       <c r="F19" s="38"/>
       <c r="L19" s="40" t="s">
+        <v>179</v>
+      </c>
+      <c r="M19" s="40" t="s">
         <v>180</v>
       </c>
-      <c r="M19" s="40" t="s">
+      <c r="N19" s="40" t="s">
         <v>181</v>
       </c>
-      <c r="N19" s="40" t="s">
+      <c r="O19" s="41" t="s">
         <v>182</v>
-      </c>
-      <c r="O19" s="41" t="s">
-        <v>183</v>
       </c>
     </row>
     <row r="20" spans="1:63" ht="15.6" customHeight="1" x14ac:dyDescent="0.2">
@@ -8082,16 +8085,16 @@
       <c r="B20" s="51"/>
       <c r="D20" s="49"/>
       <c r="L20" s="42" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="M20" s="37">
         <v>1</v>
       </c>
       <c r="N20" s="28" t="s">
+        <v>184</v>
+      </c>
+      <c r="O20" s="29" t="s">
         <v>185</v>
-      </c>
-      <c r="O20" s="29" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="21" spans="1:63" ht="15.6" customHeight="1" x14ac:dyDescent="0.2">
@@ -8099,16 +8102,16 @@
       <c r="B21" s="51"/>
       <c r="D21" s="49"/>
       <c r="L21" s="43" t="s">
+        <v>186</v>
+      </c>
+      <c r="M21" s="28" t="s">
         <v>187</v>
       </c>
-      <c r="M21" s="28" t="s">
+      <c r="N21" s="28" t="s">
+        <v>184</v>
+      </c>
+      <c r="O21" s="29" t="s">
         <v>188</v>
-      </c>
-      <c r="N21" s="28" t="s">
-        <v>185</v>
-      </c>
-      <c r="O21" s="29" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="22" spans="1:63" s="30" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.2">
@@ -8119,16 +8122,16 @@
       <c r="J22" s="32"/>
       <c r="K22" s="32"/>
       <c r="L22" s="44" t="s">
+        <v>189</v>
+      </c>
+      <c r="M22" s="28" t="s">
         <v>190</v>
       </c>
-      <c r="M22" s="28" t="s">
+      <c r="N22" s="28" t="s">
         <v>191</v>
       </c>
-      <c r="N22" s="28" t="s">
+      <c r="O22" s="29" t="s">
         <v>192</v>
-      </c>
-      <c r="O22" s="29" t="s">
-        <v>193</v>
       </c>
       <c r="P22" s="32"/>
       <c r="Q22" s="32"/>
@@ -8579,7 +8582,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="220" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B1" s="220"/>
     </row>
@@ -8588,7 +8591,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="23" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
@@ -8596,7 +8599,7 @@
         <v>1.1000000000000001</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
@@ -8604,7 +8607,7 @@
         <v>1.2</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
@@ -8612,7 +8615,7 @@
         <v>1.3</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
@@ -8620,7 +8623,7 @@
         <v>1.4</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
@@ -8628,7 +8631,7 @@
         <v>2</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
@@ -8636,7 +8639,7 @@
         <v>2.1</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
@@ -8644,7 +8647,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
@@ -8652,7 +8655,7 @@
         <v>2.2999999999999998</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
@@ -8660,7 +8663,7 @@
         <v>2.4</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
@@ -8668,7 +8671,7 @@
         <v>2.5</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
@@ -8676,7 +8679,7 @@
         <v>2.6</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
@@ -8684,7 +8687,7 @@
         <v>2.7</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
@@ -8692,7 +8695,7 @@
         <v>2.8</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
@@ -8700,7 +8703,7 @@
         <v>3</v>
       </c>
       <c r="B16" s="23" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
@@ -8708,7 +8711,7 @@
         <v>3.1</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
@@ -8716,7 +8719,7 @@
         <v>3.2</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
@@ -8724,7 +8727,7 @@
         <v>3.3</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
@@ -8732,7 +8735,7 @@
         <v>3.4</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
@@ -8740,7 +8743,7 @@
         <v>3.5</v>
       </c>
       <c r="B21" s="25" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
@@ -8748,7 +8751,7 @@
         <v>4</v>
       </c>
       <c r="B22" s="23" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
@@ -8756,7 +8759,7 @@
         <v>4.0999999999999996</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
@@ -8764,7 +8767,7 @@
         <v>4.2</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
@@ -8772,7 +8775,7 @@
         <v>4.3</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
@@ -8780,7 +8783,7 @@
         <v>4.4000000000000004</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
@@ -8788,7 +8791,7 @@
         <v>4.5999999999999996</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
@@ -8796,7 +8799,7 @@
         <v>4.7</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.2">
@@ -8804,7 +8807,7 @@
         <v>5</v>
       </c>
       <c r="B29" s="23" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
@@ -8812,7 +8815,7 @@
         <v>5.0999999999999996</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
@@ -8820,7 +8823,7 @@
         <v>5.2</v>
       </c>
       <c r="B31" s="21" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.2">
@@ -8828,7 +8831,7 @@
         <v>5.3</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.2">
@@ -8836,7 +8839,7 @@
         <v>5.4</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.2">
@@ -8844,7 +8847,7 @@
         <v>5.5</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.2">
@@ -8852,7 +8855,7 @@
         <v>5.6</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.2">
@@ -8860,7 +8863,7 @@
         <v>6</v>
       </c>
       <c r="B36" s="23" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.2">
@@ -8868,7 +8871,7 @@
         <v>6.1</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.2">
@@ -8876,7 +8879,7 @@
         <v>6.2</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.2">
@@ -8884,7 +8887,7 @@
         <v>6.3</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.2">
@@ -8892,7 +8895,7 @@
         <v>6.4</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.2">
@@ -8900,7 +8903,7 @@
         <v>6.5</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.2">
@@ -8908,7 +8911,7 @@
         <v>6.6</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.2">
@@ -8916,7 +8919,7 @@
         <v>7</v>
       </c>
       <c r="B43" s="23" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.2">
@@ -8924,7 +8927,7 @@
         <v>7.1</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.2">
@@ -8932,7 +8935,7 @@
         <v>7.2</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.2">
@@ -8940,7 +8943,7 @@
         <v>7.3</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.2">
@@ -8948,7 +8951,7 @@
         <v>7.4</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.2">
@@ -8956,7 +8959,7 @@
         <v>7.5</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.2">
@@ -8964,7 +8967,7 @@
         <v>7.6</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.2">
@@ -8972,7 +8975,7 @@
         <v>8</v>
       </c>
       <c r="B50" s="23" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.2">
@@ -8980,7 +8983,7 @@
         <v>8.1</v>
       </c>
       <c r="B51" s="20" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
   </sheetData>
@@ -9007,7 +9010,7 @@
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="221" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B1" s="222"/>
       <c r="C1" s="222"/>

</xml_diff>